<commit_message>
Track long-term memory feature in tracker + workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="350">
   <si>
     <t>Category</t>
   </si>
@@ -497,6 +497,15 @@
     <t>UPDATED Partial-&gt;Built; role-adaptation in prompt RULES</t>
   </si>
   <si>
+    <t>Long-term memory</t>
+  </si>
+  <si>
+    <t>Remembers facts (job, pets, events) + follows up across sessions</t>
+  </si>
+  <si>
+    <t>NEW; lib/memory.js, AI extraction, synced, user-forgettable</t>
+  </si>
+  <si>
     <t>Emotional Intel</t>
   </si>
   <si>
@@ -1025,7 +1034,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 124 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 125 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1497,7 +1506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2730,27 +2739,27 @@
     </row>
     <row r="62" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="C62" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="D62" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="63" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>165</v>
@@ -2765,18 +2774,18 @@
         <v>10</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>11</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>9</v>
@@ -2790,27 +2799,27 @@
     </row>
     <row r="65" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>171</v>
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>172</v>
@@ -2822,7 +2831,7 @@
         <v>9</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>174</v>
@@ -2830,7 +2839,7 @@
     </row>
     <row r="67" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>175</v>
@@ -2838,11 +2847,11 @@
       <c r="C67" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D67" s="4" t="s">
-        <v>137</v>
+      <c r="D67" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>177</v>
@@ -2850,7 +2859,7 @@
     </row>
     <row r="68" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>178</v>
@@ -2858,8 +2867,8 @@
       <c r="C68" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>9</v>
+      <c r="D68" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>55</v>
@@ -2870,13 +2879,13 @@
     </row>
     <row r="69" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="C69" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>9</v>
@@ -2885,12 +2894,12 @@
         <v>55</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="70" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>185</v>
@@ -2910,59 +2919,59 @@
     </row>
     <row r="71" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>188</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>137</v>
+        <v>189</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="72" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D72" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F72" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="73" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D73" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="E73" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>197</v>
@@ -2970,33 +2979,33 @@
     </row>
     <row r="74" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="C74" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="D74" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F74" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="75" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>9</v>
@@ -3005,12 +3014,12 @@
         <v>10</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>203</v>
+        <v>11</v>
       </c>
     </row>
     <row r="76" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>204</v>
@@ -3018,11 +3027,11 @@
       <c r="C76" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D76" s="4" t="s">
-        <v>137</v>
+      <c r="D76" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>206</v>
@@ -3030,7 +3039,7 @@
     </row>
     <row r="77" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>207</v>
@@ -3038,11 +3047,11 @@
       <c r="C77" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D77" s="3" t="s">
-        <v>9</v>
+      <c r="D77" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>209</v>
@@ -3050,7 +3059,7 @@
     </row>
     <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>210</v>
@@ -3058,19 +3067,19 @@
       <c r="C78" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D78" s="5" t="s">
-        <v>192</v>
+      <c r="D78" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>11</v>
+        <v>212</v>
       </c>
     </row>
     <row r="79" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>213</v>
@@ -3078,19 +3087,19 @@
       <c r="C79" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D79" s="4" t="s">
-        <v>137</v>
+      <c r="D79" s="5" t="s">
+        <v>195</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>215</v>
+        <v>11</v>
       </c>
     </row>
     <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>216</v>
@@ -3098,8 +3107,8 @@
       <c r="C80" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D80" s="3" t="s">
-        <v>9</v>
+      <c r="D80" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>10</v>
@@ -3110,7 +3119,7 @@
     </row>
     <row r="81" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>219</v>
@@ -3122,7 +3131,7 @@
         <v>9</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>221</v>
@@ -3130,7 +3139,7 @@
     </row>
     <row r="82" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>222</v>
@@ -3138,11 +3147,11 @@
       <c r="C82" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D82" s="4" t="s">
-        <v>137</v>
+      <c r="D82" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>224</v>
@@ -3150,7 +3159,7 @@
     </row>
     <row r="83" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>225</v>
@@ -3158,11 +3167,11 @@
       <c r="C83" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D83" s="3" t="s">
-        <v>9</v>
+      <c r="D83" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>227</v>
@@ -3170,7 +3179,7 @@
     </row>
     <row r="84" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>228</v>
@@ -3178,8 +3187,8 @@
       <c r="C84" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D84" s="5" t="s">
-        <v>192</v>
+      <c r="D84" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>55</v>
@@ -3190,7 +3199,7 @@
     </row>
     <row r="85" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>231</v>
@@ -3199,10 +3208,10 @@
         <v>232</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>233</v>
@@ -3210,27 +3219,27 @@
     </row>
     <row r="86" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="D86" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="87" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>238</v>
@@ -3242,7 +3251,7 @@
         <v>9</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>240</v>
@@ -3250,7 +3259,7 @@
     </row>
     <row r="88" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>241</v>
@@ -3265,32 +3274,32 @@
         <v>55</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
     </row>
     <row r="89" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>245</v>
+        <v>224</v>
       </c>
     </row>
     <row r="90" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>246</v>
@@ -3310,7 +3319,7 @@
     </row>
     <row r="91" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>249</v>
@@ -3318,8 +3327,8 @@
       <c r="C91" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D91" s="5" t="s">
-        <v>192</v>
+      <c r="D91" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>10</v>
@@ -3330,33 +3339,33 @@
     </row>
     <row r="92" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="C92" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="D92" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F92" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="93" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>9</v>
@@ -3370,27 +3379,27 @@
     </row>
     <row r="94" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>259</v>
+        <v>11</v>
       </c>
     </row>
     <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>260</v>
@@ -3402,21 +3411,21 @@
         <v>9</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>11</v>
+        <v>262</v>
       </c>
     </row>
     <row r="96" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>9</v>
@@ -3430,33 +3439,33 @@
     </row>
     <row r="97" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>221</v>
+        <v>11</v>
       </c>
     </row>
     <row r="98" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>9</v>
@@ -3465,18 +3474,18 @@
         <v>55</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="99" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>9</v>
@@ -3485,18 +3494,18 @@
         <v>55</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>52</v>
+        <v>224</v>
       </c>
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>9</v>
@@ -3510,19 +3519,19 @@
     </row>
     <row r="101" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>193</v>
+        <v>55</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>52</v>
@@ -3530,39 +3539,39 @@
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="D102" s="5" t="s">
-        <v>192</v>
+        <v>276</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>11</v>
@@ -3570,7 +3579,7 @@
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>278</v>
+        <v>255</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>279</v>
@@ -3578,19 +3587,19 @@
       <c r="C104" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="D104" s="3" t="s">
-        <v>9</v>
+      <c r="D104" s="5" t="s">
+        <v>195</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>55</v>
+        <v>196</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>281</v>
+        <v>11</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>282</v>
@@ -3602,35 +3611,35 @@
         <v>9</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>193</v>
+        <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>221</v>
+        <v>284</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>55</v>
+        <v>196</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>286</v>
+        <v>224</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>287</v>
@@ -3642,7 +3651,7 @@
         <v>9</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>193</v>
+        <v>55</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>289</v>
@@ -3650,7 +3659,7 @@
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>290</v>
@@ -3662,47 +3671,47 @@
         <v>9</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>55</v>
+        <v>196</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>192</v>
+        <v>294</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>193</v>
+        <v>55</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>11</v>
+        <v>224</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D110" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>11</v>
@@ -3710,7 +3719,7 @@
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>297</v>
@@ -3718,19 +3727,19 @@
       <c r="C111" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="D111" s="3" t="s">
-        <v>9</v>
+      <c r="D111" s="5" t="s">
+        <v>195</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>10</v>
+        <v>196</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>299</v>
+        <v>11</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>300</v>
@@ -3742,7 +3751,7 @@
         <v>9</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>302</v>
@@ -3750,7 +3759,7 @@
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>303</v>
@@ -3758,11 +3767,11 @@
       <c r="C113" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="D113" s="4" t="s">
-        <v>137</v>
+      <c r="D113" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>305</v>
@@ -3770,7 +3779,7 @@
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>306</v>
@@ -3778,31 +3787,31 @@
       <c r="C114" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="D114" s="5" t="s">
-        <v>192</v>
+      <c r="D114" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>193</v>
+        <v>10</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>11</v>
+        <v>308</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D115" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F115" s="2" t="s">
         <v>11</v>
@@ -3810,7 +3819,7 @@
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>311</v>
@@ -3818,19 +3827,19 @@
       <c r="C116" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="D116" s="3" t="s">
-        <v>9</v>
+      <c r="D116" s="5" t="s">
+        <v>195</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>10</v>
+        <v>196</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>313</v>
+        <v>11</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>314</v>
@@ -3850,7 +3859,7 @@
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>317</v>
@@ -3865,38 +3874,38 @@
         <v>10</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>52</v>
+        <v>319</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>221</v>
+        <v>52</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>9</v>
@@ -3905,18 +3914,18 @@
         <v>55</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
@@ -3925,32 +3934,32 @@
         <v>55</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>52</v>
+        <v>224</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="D122" s="4" t="s">
-        <v>137</v>
+        <v>327</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>327</v>
+        <v>52</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>328</v>
@@ -3958,39 +3967,39 @@
       <c r="C123" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="D123" s="3" t="s">
-        <v>9</v>
+      <c r="D123" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>52</v>
+        <v>330</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="D124" s="4" t="s">
-        <v>137</v>
+        <v>332</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>332</v>
+        <v>52</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>333</v>
@@ -3998,8 +4007,8 @@
       <c r="C125" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D125" s="5" t="s">
-        <v>192</v>
+      <c r="D125" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>55</v>
@@ -4008,8 +4017,28 @@
         <v>335</v>
       </c>
     </row>
+    <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F125"/>
+  <autoFilter ref="A1:F126"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4026,17 +4055,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4044,10 +4073,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4055,10 +4084,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4069,34 +4098,34 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B8">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B9" s="13">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4110,10 +4139,10 @@
         <v>137</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4206,7 +4235,7 @@
         <v>139</v>
       </c>
       <c r="B18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -4215,12 +4244,12 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -4237,7 +4266,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -4254,7 +4283,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -4271,7 +4300,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -4288,7 +4317,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B23">
         <v>5</v>
@@ -4305,7 +4334,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B24">
         <v>10</v>
@@ -4322,7 +4351,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4339,7 +4368,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4356,7 +4385,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Track proactive follow-ups + away-recap in tracker/workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="355">
   <si>
     <t>Category</t>
   </si>
@@ -353,6 +353,24 @@
     <t>UPDATED Future-&gt;Built; NEW proactive</t>
   </si>
   <si>
+    <t>Proactive memory follow-ups</t>
+  </si>
+  <si>
+    <t>Companions ask how a remembered past event went, deduped</t>
+  </si>
+  <si>
+    <t>NEW; pendingFollowups/markFollowed, return + idle</t>
+  </si>
+  <si>
+    <t>While-you-were-away recap</t>
+  </si>
+  <si>
+    <t>Labeled ambient catch-up divider on open</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
     <t>Companion disagreements</t>
   </si>
   <si>
@@ -602,9 +620,6 @@
     <t>Future</t>
   </si>
   <si>
-    <t>P2</t>
-  </si>
-  <si>
     <t>On-device only by design</t>
   </si>
   <si>
@@ -1034,7 +1049,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 125 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 127 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1052,7 +1067,7 @@
     <t>7%</t>
   </si>
   <si>
-    <t>10%</t>
+    <t>9%</t>
   </si>
   <si>
     <t>Total</t>
@@ -1506,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2391,10 +2406,10 @@
         <v>9</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2402,19 +2417,19 @@
         <v>105</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2422,10 +2437,10 @@
         <v>105</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>9</v>
@@ -2434,7 +2449,7 @@
         <v>10</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>120</v>
+        <v>11</v>
       </c>
     </row>
     <row r="47" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2451,10 +2466,10 @@
         <v>9</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2462,19 +2477,19 @@
         <v>105</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2482,19 +2497,19 @@
         <v>105</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>127</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2502,19 +2517,19 @@
         <v>105</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2522,19 +2537,19 @@
         <v>105</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="52" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2542,10 +2557,10 @@
         <v>105</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>9</v>
@@ -2562,13 +2577,13 @@
         <v>105</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D53" s="4" t="s">
         <v>137</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>55</v>
@@ -2579,13 +2594,13 @@
     </row>
     <row r="54" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>9</v>
@@ -2599,19 +2614,19 @@
     </row>
     <row r="55" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="D55" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="E55" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>144</v>
@@ -2619,27 +2634,27 @@
     </row>
     <row r="56" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>147</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>148</v>
@@ -2654,38 +2669,38 @@
         <v>10</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>11</v>
+        <v>150</v>
       </c>
     </row>
     <row r="58" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>11</v>
+        <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>9</v>
@@ -2694,32 +2709,32 @@
         <v>10</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>154</v>
+        <v>11</v>
       </c>
     </row>
     <row r="60" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>157</v>
+        <v>11</v>
       </c>
     </row>
     <row r="61" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>158</v>
@@ -2739,7 +2754,7 @@
     </row>
     <row r="62" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>161</v>
@@ -2751,7 +2766,7 @@
         <v>9</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>163</v>
@@ -2759,53 +2774,53 @@
     </row>
     <row r="63" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="C63" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="D63" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="64" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="D64" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="65" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>9</v>
@@ -2814,38 +2829,38 @@
         <v>10</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>11</v>
+        <v>173</v>
       </c>
     </row>
     <row r="66" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>174</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>9</v>
@@ -2854,12 +2869,12 @@
         <v>10</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>177</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>178</v>
@@ -2867,8 +2882,8 @@
       <c r="C68" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D68" s="4" t="s">
-        <v>137</v>
+      <c r="D68" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>55</v>
@@ -2879,7 +2894,7 @@
     </row>
     <row r="69" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>181</v>
@@ -2891,7 +2906,7 @@
         <v>9</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>183</v>
@@ -2899,33 +2914,33 @@
     </row>
     <row r="70" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="C70" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>9</v>
+      <c r="D70" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>9</v>
@@ -2934,112 +2949,112 @@
         <v>55</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="72" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>191</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>137</v>
+        <v>192</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="73" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D73" s="5" t="s">
         <v>195</v>
       </c>
+      <c r="D73" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E73" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="74" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>9</v>
+        <v>185</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="75" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D75" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="E75" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="76" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="D76" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F76" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="77" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>207</v>
@@ -3047,145 +3062,145 @@
       <c r="C77" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D77" s="4" t="s">
-        <v>137</v>
+      <c r="D77" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>209</v>
+        <v>11</v>
       </c>
     </row>
     <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="D78" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="79" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>195</v>
+      <c r="D79" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>11</v>
+        <v>214</v>
       </c>
     </row>
     <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="C80" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="D80" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F80" s="2" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B81" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C81" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>9</v>
+      <c r="D81" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>221</v>
+        <v>11</v>
       </c>
     </row>
     <row r="82" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="D82" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="83" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="D83" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="D83" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="84" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B84" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C84" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>229</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>9</v>
@@ -3194,112 +3209,112 @@
         <v>55</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="85" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B85" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="D85" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F85" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="D85" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="86" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B86" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="D86" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="D86" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="87" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C87" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="D87" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F87" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="88" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>237</v>
+        <v>220</v>
       </c>
       <c r="B88" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F88" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F88" s="2" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="89" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B89" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C89" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="D89" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F89" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="90" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>246</v>
@@ -3311,7 +3326,7 @@
         <v>9</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>248</v>
@@ -3319,7 +3334,7 @@
     </row>
     <row r="91" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>249</v>
@@ -3331,95 +3346,95 @@
         <v>9</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>251</v>
+        <v>229</v>
       </c>
     </row>
     <row r="92" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B92" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C92" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="D92" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F92" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="D92" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="93" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C93" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="D93" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F93" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E93" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F93" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="94" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="B94" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="D94" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>262</v>
+        <v>11</v>
       </c>
     </row>
     <row r="96" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>263</v>
@@ -3439,7 +3454,7 @@
     </row>
     <row r="97" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>265</v>
@@ -3451,61 +3466,61 @@
         <v>9</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>11</v>
+        <v>267</v>
       </c>
     </row>
     <row r="98" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>224</v>
+        <v>11</v>
       </c>
     </row>
     <row r="99" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>224</v>
+        <v>11</v>
       </c>
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>9</v>
@@ -3514,18 +3529,18 @@
         <v>55</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>52</v>
+        <v>229</v>
       </c>
     </row>
     <row r="101" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>9</v>
@@ -3534,24 +3549,24 @@
         <v>55</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>52</v>
+        <v>229</v>
       </c>
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>196</v>
+        <v>55</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>52</v>
@@ -3559,47 +3574,47 @@
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="D103" s="5" t="s">
-        <v>195</v>
+        <v>279</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>196</v>
+        <v>55</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>195</v>
+        <v>281</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>282</v>
@@ -3607,39 +3622,39 @@
       <c r="C105" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D105" s="3" t="s">
-        <v>9</v>
+      <c r="D105" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>284</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="B106" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C106" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="C106" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D106" s="3" t="s">
-        <v>9</v>
+      <c r="D106" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>224</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>287</v>
@@ -3659,7 +3674,7 @@
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>290</v>
@@ -3671,21 +3686,21 @@
         <v>9</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>292</v>
+        <v>229</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B109" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>294</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>9</v>
@@ -3694,12 +3709,12 @@
         <v>55</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>224</v>
+        <v>294</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>295</v>
@@ -3707,39 +3722,39 @@
       <c r="C110" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D110" s="5" t="s">
-        <v>195</v>
+      <c r="D110" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>11</v>
+        <v>297</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>195</v>
+        <v>299</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>196</v>
+        <v>55</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>11</v>
+        <v>229</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>300</v>
@@ -3747,79 +3762,79 @@
       <c r="C112" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="D112" s="3" t="s">
-        <v>9</v>
+      <c r="D112" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>302</v>
+        <v>11</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B113" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C113" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="C113" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D113" s="3" t="s">
-        <v>9</v>
+      <c r="D113" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>305</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B114" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C114" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="C114" s="2" t="s">
+      <c r="D114" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F114" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="D114" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B115" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C115" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="C115" s="2" t="s">
+      <c r="D115" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F115" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="F115" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>311</v>
@@ -3827,19 +3842,19 @@
       <c r="C116" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="D116" s="5" t="s">
-        <v>195</v>
+      <c r="D116" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>196</v>
+        <v>10</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>11</v>
+        <v>313</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>314</v>
@@ -3847,59 +3862,59 @@
       <c r="C117" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D117" s="3" t="s">
-        <v>9</v>
+      <c r="D117" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>316</v>
+        <v>11</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="C118" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>9</v>
+      <c r="D118" s="5" t="s">
+        <v>201</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>319</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B119" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C119" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C119" s="2" t="s">
+      <c r="D119" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F119" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F119" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>322</v>
@@ -3911,41 +3926,41 @@
         <v>9</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>224</v>
+        <v>324</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>224</v>
+        <v>52</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
@@ -3954,32 +3969,32 @@
         <v>55</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>52</v>
+        <v>229</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D123" s="4" t="s">
-        <v>137</v>
+        <v>330</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>330</v>
+        <v>229</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>331</v>
@@ -3999,7 +4014,7 @@
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>333</v>
@@ -4008,7 +4023,7 @@
         <v>334</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>55</v>
@@ -4019,7 +4034,7 @@
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>336</v>
@@ -4027,18 +4042,58 @@
       <c r="C126" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="D126" s="5" t="s">
-        <v>195</v>
+      <c r="D126" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F126" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>338</v>
       </c>
+      <c r="C127" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>343</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F126"/>
+  <autoFilter ref="A1:F128"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4055,17 +4110,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4073,10 +4128,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4084,48 +4139,48 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B7">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B8">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B9" s="13">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4136,13 +4191,13 @@
         <v>9</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4218,7 +4273,7 @@
         <v>105</v>
       </c>
       <c r="B17">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -4227,12 +4282,12 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B18">
         <v>9</v>
@@ -4249,7 +4304,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -4266,7 +4321,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -4283,7 +4338,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -4300,7 +4355,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -4317,7 +4372,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B23">
         <v>5</v>
@@ -4334,7 +4389,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B24">
         <v>10</v>
@@ -4351,7 +4406,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4368,7 +4423,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4385,7 +4440,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
AI disclosure: one-time ack gate + once-daily in-chat reminder
Per the request, the disclosure now has two parts instead of an hourly note:
- A blocking, must-click "I understand" gate shown once ever, the first time
  the user reaches chat (after accepting Terms + Privacy on Welcome). Persisted
  via localStorage so it never reappears.
- A gentle in-chat reminder shown at most once per calendar day thereafter
  (the ack covers day one). Still required and not user-disableable.

- disclosure.js: isAcknowledged/acknowledgeDisclosure + consumeDailyReminder
  (date-stamped, fires once/day); dropped the hourly accumulator.
- Chat.jsx: DisclosureGate overlay component + needsAck state; mount logic now
  appends the reminder only when acknowledged AND not already shown today.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -662,10 +662,10 @@
     <t>AI disclosure reminders</t>
   </si>
   <si>
-    <t>Required, recurring, not disableable</t>
-  </si>
-  <si>
-    <t>NEW; ToS 13; open + hourly</t>
+    <t>One-time must-click ack at start + once-daily in-chat reminder</t>
+  </si>
+  <si>
+    <t>UPDATED; ToS 13; ack gate + daily, not disableable</t>
   </si>
   <si>
     <t>Multi-companion explicit</t>

</xml_diff>

<commit_message>
Add generative companion avatars + custom colour wheel
Avatars: each companion gets a unique "cosmic sigil" — a deterministic
constellation of stars plus a tilted orbital ring over their colour gradient,
seeded by identity (components/Avatar.jsx). Pure SVG: no uploads, no network,
no image-AI cost; recolours instantly. Replaces the plain colour dots in chat
bubbles, both chat headers, the companion picker, the unlock sheet, and the
profile hero. WakingUp keeps its formless pulse so the sigil "resolves" on wake.

Colour wheel: the profile Appearance section now has a custom colour picker
(<input type="color">) alongside the 8 presets, so a companion can be any
colour. Seed is identity-only, so recolouring re-tints the same sigil rather
than reshuffling it. Custom colour persists + cloud-syncs like the presets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="361">
   <si>
     <t>Category</t>
   </si>
@@ -818,13 +818,22 @@
     <t>Abstract color per companion</t>
   </si>
   <si>
+    <t>Generative avatars</t>
+  </si>
+  <si>
+    <t>Unique cosmic constellation sigil per companion</t>
+  </si>
+  <si>
+    <t>NEW; components/Avatar.jsx, deterministic SVG, recolors live</t>
+  </si>
+  <si>
     <t>Cosmetic customization</t>
   </si>
   <si>
-    <t>Recolor a companion (8-color palette)</t>
-  </si>
-  <si>
-    <t>NEW; ToS 4.1 free tier</t>
+    <t>Recolor a companion: 8-color palette + custom color wheel</t>
+  </si>
+  <si>
+    <t>UPDATED; ToS 4.1; &lt;input type=color&gt; any color</t>
   </si>
   <si>
     <t>Animated waking sequence</t>
@@ -1058,7 +1067,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 128 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 129 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1530,7 +1539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3515,10 +3524,10 @@
         <v>9</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>11</v>
+        <v>273</v>
       </c>
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3526,10 +3535,10 @@
         <v>263</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>9</v>
@@ -3546,19 +3555,19 @@
         <v>263</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3566,10 +3575,10 @@
         <v>263</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>9</v>
@@ -3586,10 +3595,10 @@
         <v>263</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>9</v>
@@ -3598,7 +3607,7 @@
         <v>55</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3606,10 +3615,10 @@
         <v>263</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>9</v>
@@ -3626,16 +3635,16 @@
         <v>263</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>52</v>
@@ -3646,19 +3655,19 @@
         <v>263</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>204</v>
+        <v>287</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3666,10 +3675,10 @@
         <v>263</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>204</v>
@@ -3683,7 +3692,7 @@
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>289</v>
+        <v>263</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>290</v>
@@ -3691,19 +3700,19 @@
       <c r="C108" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="D108" s="3" t="s">
-        <v>9</v>
+      <c r="D108" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>292</v>
+        <v>11</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>293</v>
@@ -3715,35 +3724,35 @@
         <v>9</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>232</v>
+        <v>295</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>298</v>
@@ -3755,7 +3764,7 @@
         <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>300</v>
@@ -3763,7 +3772,7 @@
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>301</v>
@@ -3775,41 +3784,41 @@
         <v>9</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>232</v>
+        <v>303</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>204</v>
+        <v>305</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>11</v>
+        <v>232</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>204</v>
@@ -3823,7 +3832,7 @@
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>308</v>
@@ -3831,19 +3840,19 @@
       <c r="C115" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D115" s="3" t="s">
-        <v>9</v>
+      <c r="D115" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>310</v>
+        <v>11</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>311</v>
@@ -3855,7 +3864,7 @@
         <v>9</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>313</v>
@@ -3863,7 +3872,7 @@
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>314</v>
@@ -3871,11 +3880,11 @@
       <c r="C117" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D117" s="4" t="s">
-        <v>146</v>
+      <c r="D117" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>316</v>
@@ -3883,7 +3892,7 @@
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>317</v>
@@ -3891,25 +3900,25 @@
       <c r="C118" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>204</v>
+      <c r="D118" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>11</v>
+        <v>319</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>204</v>
@@ -3923,7 +3932,7 @@
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>322</v>
@@ -3931,19 +3940,19 @@
       <c r="C120" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="D120" s="3" t="s">
-        <v>9</v>
+      <c r="D120" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>324</v>
+        <v>11</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>325</v>
@@ -3963,7 +3972,7 @@
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>328</v>
@@ -3978,38 +3987,38 @@
         <v>10</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>52</v>
+        <v>330</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>232</v>
+        <v>52</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>9</v>
@@ -4023,13 +4032,13 @@
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>9</v>
@@ -4038,32 +4047,32 @@
         <v>55</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="D126" s="4" t="s">
-        <v>146</v>
+        <v>338</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>338</v>
+        <v>52</v>
       </c>
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>339</v>
@@ -4071,39 +4080,39 @@
       <c r="C127" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="D127" s="3" t="s">
-        <v>9</v>
+      <c r="D127" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>52</v>
+        <v>341</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="D128" s="4" t="s">
-        <v>146</v>
+        <v>343</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>343</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>344</v>
@@ -4111,8 +4120,8 @@
       <c r="C129" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="D129" s="5" t="s">
-        <v>204</v>
+      <c r="D129" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>55</v>
@@ -4121,8 +4130,28 @@
         <v>346</v>
       </c>
     </row>
+    <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F129"/>
+  <autoFilter ref="A1:F130"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4139,17 +4168,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4157,10 +4186,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4168,10 +4197,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4182,7 +4211,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4193,23 +4222,23 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B9" s="13">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4226,7 +4255,7 @@
         <v>204</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4421,7 +4450,7 @@
         <v>263</v>
       </c>
       <c r="B24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -4430,12 +4459,12 @@
         <v>2</v>
       </c>
       <c r="E24">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4452,7 +4481,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4469,7 +4498,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Log future feature: lounge decoration
Track a user request to customize the sitting space with background pictures,
tiles, and patterns/themes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="367">
   <si>
     <t>Category</t>
   </si>
@@ -836,6 +836,15 @@
     <t>NEW; screens/CompanionSpace.jsx, positions persist+sync</t>
   </si>
   <si>
+    <t>Lounge decoration</t>
+  </si>
+  <si>
+    <t>Customize the Space: background pictures, tiles, patterns/themes</t>
+  </si>
+  <si>
+    <t>User request; decorate the sitting space (uploads or preset patterns)</t>
+  </si>
+  <si>
     <t>Cosmetic customization</t>
   </si>
   <si>
@@ -1076,7 +1085,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 130 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 131 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1088,13 +1097,13 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>84%</t>
+    <t>83%</t>
   </si>
   <si>
     <t>7%</t>
   </si>
   <si>
-    <t>9%</t>
+    <t>10%</t>
   </si>
   <si>
     <t>Total</t>
@@ -1548,7 +1557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3549,11 +3558,11 @@
       <c r="C100" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D100" s="3" t="s">
-        <v>9</v>
+      <c r="D100" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>276</v>
@@ -3573,10 +3582,10 @@
         <v>9</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>11</v>
+        <v>279</v>
       </c>
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3584,10 +3593,10 @@
         <v>263</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>9</v>
@@ -3604,19 +3613,19 @@
         <v>263</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3624,10 +3633,10 @@
         <v>263</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>9</v>
@@ -3644,10 +3653,10 @@
         <v>263</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
@@ -3656,7 +3665,7 @@
         <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3664,10 +3673,10 @@
         <v>263</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
@@ -3684,16 +3693,16 @@
         <v>263</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>52</v>
@@ -3704,19 +3713,19 @@
         <v>263</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>204</v>
+        <v>293</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3724,10 +3733,10 @@
         <v>263</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>204</v>
@@ -3741,7 +3750,7 @@
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>295</v>
+        <v>263</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>296</v>
@@ -3749,19 +3758,19 @@
       <c r="C110" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D110" s="3" t="s">
-        <v>9</v>
+      <c r="D110" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>298</v>
+        <v>11</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>299</v>
@@ -3773,35 +3782,35 @@
         <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>232</v>
+        <v>301</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>303</v>
+        <v>232</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>304</v>
@@ -3813,7 +3822,7 @@
         <v>9</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>306</v>
@@ -3821,7 +3830,7 @@
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>307</v>
@@ -3833,41 +3842,41 @@
         <v>9</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>232</v>
+        <v>309</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>204</v>
+        <v>311</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>11</v>
+        <v>232</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>204</v>
@@ -3881,7 +3890,7 @@
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>314</v>
@@ -3889,19 +3898,19 @@
       <c r="C117" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D117" s="3" t="s">
-        <v>9</v>
+      <c r="D117" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>316</v>
+        <v>11</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>317</v>
@@ -3913,7 +3922,7 @@
         <v>9</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>319</v>
@@ -3921,7 +3930,7 @@
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>320</v>
@@ -3929,11 +3938,11 @@
       <c r="C119" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D119" s="4" t="s">
-        <v>146</v>
+      <c r="D119" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>322</v>
@@ -3941,7 +3950,7 @@
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>323</v>
@@ -3949,25 +3958,25 @@
       <c r="C120" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D120" s="5" t="s">
-        <v>204</v>
+      <c r="D120" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>11</v>
+        <v>325</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>204</v>
@@ -3981,7 +3990,7 @@
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>328</v>
@@ -3989,19 +3998,19 @@
       <c r="C122" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="D122" s="3" t="s">
-        <v>9</v>
+      <c r="D122" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>330</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>331</v>
@@ -4021,7 +4030,7 @@
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>334</v>
@@ -4036,38 +4045,38 @@
         <v>10</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>52</v>
+        <v>336</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>232</v>
+        <v>52</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>9</v>
@@ -4081,13 +4090,13 @@
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>9</v>
@@ -4096,32 +4105,32 @@
         <v>55</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="D128" s="4" t="s">
-        <v>146</v>
+        <v>344</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>344</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>345</v>
@@ -4129,39 +4138,39 @@
       <c r="C129" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="D129" s="3" t="s">
-        <v>9</v>
+      <c r="D129" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>52</v>
+        <v>347</v>
       </c>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="D130" s="4" t="s">
-        <v>146</v>
+        <v>349</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>349</v>
+        <v>52</v>
       </c>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>350</v>
@@ -4169,8 +4178,8 @@
       <c r="C131" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="D131" s="5" t="s">
-        <v>204</v>
+      <c r="D131" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>55</v>
@@ -4179,8 +4188,28 @@
         <v>352</v>
       </c>
     </row>
+    <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F131"/>
+  <autoFilter ref="A1:F132"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4197,17 +4226,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4215,10 +4244,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4229,7 +4258,7 @@
         <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4240,7 +4269,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4248,26 +4277,26 @@
         <v>204</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B9" s="13">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4284,7 +4313,7 @@
         <v>204</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4485,15 +4514,15 @@
         <v>0</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E24">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4510,7 +4539,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4527,7 +4556,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Space: approach-on-talk animation + personality pet reactions
- Approach animation: when two companions trade ambient lines, the pair now
  leans ~38% toward each other (smooth left/top easing) and glows, plays the
  exchange as a timed back-and-forth of bubbles, then drifts back when done.
- Personality pet reactions: petStyle() reads each companion's personality,
  quirk, and builder traits to choose the pet response — playful giggles,
  shy "oh—", warm "mmm♡", dry "…heh", or energetic "YES!" — with matching
  particle emojis, a floating reaction word, and burst size.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="373">
   <si>
     <t>Category</t>
   </si>
@@ -836,6 +836,24 @@
     <t>NEW; screens/CompanionSpace.jsx, positions persist+sync</t>
   </si>
   <si>
+    <t>Space approach animation</t>
+  </si>
+  <si>
+    <t>Talking companions lean toward each other + trade lines</t>
+  </si>
+  <si>
+    <t>NEW; pair leans in during ambient exchange</t>
+  </si>
+  <si>
+    <t>Personality pet reactions</t>
+  </si>
+  <si>
+    <t>Pet response (emoji/word/burst) varies by personality</t>
+  </si>
+  <si>
+    <t>NEW; petStyle() from personality+traits</t>
+  </si>
+  <si>
     <t>Lounge decoration</t>
   </si>
   <si>
@@ -1085,7 +1103,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 131 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 133 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1557,7 +1575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3558,8 +3576,8 @@
       <c r="C100" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D100" s="5" t="s">
-        <v>204</v>
+      <c r="D100" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>118</v>
@@ -3582,7 +3600,7 @@
         <v>9</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>279</v>
@@ -3598,14 +3616,14 @@
       <c r="C102" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D102" s="3" t="s">
-        <v>9</v>
+      <c r="D102" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>11</v>
+        <v>282</v>
       </c>
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3613,19 +3631,19 @@
         <v>263</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>11</v>
+        <v>285</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3633,19 +3651,19 @@
         <v>263</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3653,19 +3671,19 @@
         <v>263</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3673,10 +3691,10 @@
         <v>263</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
@@ -3685,7 +3703,7 @@
         <v>55</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3693,10 +3711,10 @@
         <v>263</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
@@ -3705,7 +3723,7 @@
         <v>55</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3713,16 +3731,16 @@
         <v>263</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>52</v>
@@ -3733,19 +3751,19 @@
         <v>263</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>204</v>
+        <v>297</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3753,44 +3771,44 @@
         <v>263</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>204</v>
+        <v>299</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>298</v>
+        <v>263</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>9</v>
+        <v>301</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>301</v>
+        <v>11</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>298</v>
+        <v>263</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>302</v>
@@ -3798,25 +3816,25 @@
       <c r="C112" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D112" s="3" t="s">
-        <v>9</v>
+      <c r="D112" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>9</v>
@@ -3825,18 +3843,18 @@
         <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>9</v>
@@ -3845,12 +3863,12 @@
         <v>118</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>309</v>
+        <v>232</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>310</v>
@@ -3865,72 +3883,72 @@
         <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>232</v>
+        <v>312</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>204</v>
+        <v>314</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>11</v>
+        <v>315</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="D117" s="5" t="s">
-        <v>204</v>
+        <v>317</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>11</v>
+        <v>232</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>9</v>
+        <v>319</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>319</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>320</v>
@@ -3938,19 +3956,19 @@
       <c r="C119" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D119" s="3" t="s">
-        <v>9</v>
+      <c r="D119" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>322</v>
+        <v>11</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>323</v>
@@ -3958,8 +3976,8 @@
       <c r="C120" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D120" s="4" t="s">
-        <v>146</v>
+      <c r="D120" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>10</v>
@@ -3970,7 +3988,7 @@
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>326</v>
@@ -3978,59 +3996,59 @@
       <c r="C121" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="D121" s="5" t="s">
-        <v>204</v>
+      <c r="D121" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>11</v>
+        <v>328</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>204</v>
+        <v>330</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>11</v>
+        <v>331</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="D123" s="3" t="s">
-        <v>9</v>
+        <v>333</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>333</v>
+        <v>11</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>334</v>
@@ -4038,19 +4056,19 @@
       <c r="C124" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D124" s="3" t="s">
-        <v>9</v>
+      <c r="D124" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>336</v>
+        <v>11</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>337</v>
@@ -4065,58 +4083,58 @@
         <v>10</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>52</v>
+        <v>339</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>232</v>
+        <v>342</v>
       </c>
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>232</v>
+        <v>52</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>9</v>
@@ -4125,38 +4143,38 @@
         <v>55</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="D129" s="4" t="s">
-        <v>146</v>
+        <v>348</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>347</v>
+        <v>232</v>
       </c>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4170,13 +4188,13 @@
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>146</v>
@@ -4185,31 +4203,71 @@
         <v>55</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="D132" s="5" t="s">
-        <v>204</v>
+        <v>355</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>355</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="D133" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>361</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F132"/>
+  <autoFilter ref="A1:F134"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4226,17 +4284,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4244,10 +4302,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4255,10 +4313,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C6" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4269,7 +4327,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4280,23 +4338,23 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B9" s="13">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4313,7 +4371,7 @@
         <v>204</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4508,7 +4566,7 @@
         <v>263</v>
       </c>
       <c r="B24">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -4517,12 +4575,12 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4539,7 +4597,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4556,7 +4614,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Add companion presence ("right now" activity)
Companions now feel like they have lives of their own: each shows a light,
personality-flavoured sense of what they're up to ("chasing a melody",
"thinking about you", "down a rabbit hole"). Deterministic per companion +
~40-min time bucket, so it's stable within a sitting and free (no API).

- lib/presence.js: currentActivity(comp) — trait-detected pool blended with
  generic + occasional "thinking about you"; sleeping reads as "resting".
- Shown under each avatar in the Space (when not mid-conversation) and as a
  "Right now" card on the companion profile.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="376">
   <si>
     <t>Category</t>
   </si>
@@ -854,6 +854,15 @@
     <t>NEW; petStyle() from personality+traits</t>
   </si>
   <si>
+    <t>Companion presence</t>
+  </si>
+  <si>
+    <t>"Right now" activity per companion (lives of their own)</t>
+  </si>
+  <si>
+    <t>NEW; lib/presence.js, shown in Space + profile, time-bucketed</t>
+  </si>
+  <si>
     <t>Lounge decoration</t>
   </si>
   <si>
@@ -1103,7 +1112,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 133 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 134 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1115,7 +1124,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>83%</t>
+    <t>84%</t>
   </si>
   <si>
     <t>7%</t>
@@ -1575,7 +1584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3608,7 +3617,7 @@
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>263</v>
+        <v>148</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>280</v>
@@ -3616,8 +3625,8 @@
       <c r="C102" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D102" s="5" t="s">
-        <v>204</v>
+      <c r="D102" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>118</v>
@@ -3636,11 +3645,11 @@
       <c r="C103" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D103" s="3" t="s">
-        <v>9</v>
+      <c r="D103" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>285</v>
@@ -3660,10 +3669,10 @@
         <v>9</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>11</v>
+        <v>288</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3671,10 +3680,10 @@
         <v>263</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
@@ -3691,19 +3700,19 @@
         <v>263</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3711,10 +3720,10 @@
         <v>263</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
@@ -3731,10 +3740,10 @@
         <v>263</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>9</v>
@@ -3743,7 +3752,7 @@
         <v>55</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3751,10 +3760,10 @@
         <v>263</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>9</v>
@@ -3771,16 +3780,16 @@
         <v>263</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>52</v>
@@ -3791,19 +3800,19 @@
         <v>263</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>204</v>
+        <v>302</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3811,10 +3820,10 @@
         <v>263</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>204</v>
@@ -3828,7 +3837,7 @@
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>304</v>
+        <v>263</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>305</v>
@@ -3836,19 +3845,19 @@
       <c r="C113" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D113" s="3" t="s">
-        <v>9</v>
+      <c r="D113" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>307</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>308</v>
@@ -3860,35 +3869,35 @@
         <v>9</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>232</v>
+        <v>310</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>312</v>
+        <v>232</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>313</v>
@@ -3900,7 +3909,7 @@
         <v>9</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>315</v>
@@ -3908,7 +3917,7 @@
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>316</v>
@@ -3920,41 +3929,41 @@
         <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>232</v>
+        <v>318</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>204</v>
+        <v>320</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>11</v>
+        <v>232</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>204</v>
@@ -3968,7 +3977,7 @@
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>323</v>
@@ -3976,19 +3985,19 @@
       <c r="C120" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D120" s="3" t="s">
-        <v>9</v>
+      <c r="D120" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>325</v>
+        <v>11</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>326</v>
@@ -4000,7 +4009,7 @@
         <v>9</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>328</v>
@@ -4008,7 +4017,7 @@
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>329</v>
@@ -4016,11 +4025,11 @@
       <c r="C122" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="D122" s="4" t="s">
-        <v>146</v>
+      <c r="D122" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>331</v>
@@ -4028,7 +4037,7 @@
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>332</v>
@@ -4036,25 +4045,25 @@
       <c r="C123" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D123" s="5" t="s">
-        <v>204</v>
+      <c r="D123" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>11</v>
+        <v>334</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>204</v>
@@ -4068,7 +4077,7 @@
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>337</v>
@@ -4076,19 +4085,19 @@
       <c r="C125" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D125" s="3" t="s">
-        <v>9</v>
+      <c r="D125" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>339</v>
+        <v>11</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>340</v>
@@ -4108,7 +4117,7 @@
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>343</v>
@@ -4123,38 +4132,38 @@
         <v>10</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>52</v>
+        <v>345</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>232</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>9</v>
@@ -4168,13 +4177,13 @@
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4183,32 +4192,32 @@
         <v>55</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>52</v>
+        <v>232</v>
       </c>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="D131" s="4" t="s">
-        <v>146</v>
+        <v>353</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>353</v>
+        <v>52</v>
       </c>
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>354</v>
@@ -4216,39 +4225,39 @@
       <c r="C132" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="D132" s="3" t="s">
-        <v>9</v>
+      <c r="D132" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>52</v>
+        <v>356</v>
       </c>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="D133" s="4" t="s">
-        <v>146</v>
+        <v>358</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>358</v>
+        <v>52</v>
       </c>
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>359</v>
@@ -4256,8 +4265,8 @@
       <c r="C134" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="D134" s="5" t="s">
-        <v>204</v>
+      <c r="D134" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>55</v>
@@ -4266,8 +4275,28 @@
         <v>361</v>
       </c>
     </row>
+    <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>364</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F134"/>
+  <autoFilter ref="A1:F135"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4284,17 +4313,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4302,10 +4331,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4313,10 +4342,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4327,7 +4356,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4338,23 +4367,23 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B9" s="13">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4371,7 +4400,7 @@
         <v>204</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4464,7 +4493,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -4473,7 +4502,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4580,7 +4609,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4597,7 +4626,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4614,7 +4643,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Add ambient conversation alerts (push)
Push check-ins now sometimes ping the user that their companions were chatting
with each other ("Maya and Sam were just talking about you ✦"), drawing them
back to catch the moment. Fires ~40% of the time when 2+ companions are awake
and there's no pending memory follow-up; respects the existing check-in
schedule/enable.

- worker.js: ambientAlertLine() variants; cron prefers followup > ambient
  alert > generic check-in; gated by blob.ambientAlerts (default on).
- Settings: "Conversation alerts" toggle under Notifications.
- ambientAlerts state plumbed through Chat persistence + App resume/sync.

Auto-deploys to the worker via GitHub Actions on push. Server tests pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="377">
   <si>
     <t>Category</t>
   </si>
@@ -980,7 +980,10 @@
     <t>Ambient conversation alerts</t>
   </si>
   <si>
-    <t>Notified companions were chatting</t>
+    <t>Push when companions were chatting with each other</t>
+  </si>
+  <si>
+    <t>NEW; cron ambientAlertLine, Settings toggle, default on</t>
   </si>
   <si>
     <t>Location-based nudges</t>
@@ -1130,7 +1133,7 @@
     <t>7%</t>
   </si>
   <si>
-    <t>10%</t>
+    <t>9%</t>
   </si>
   <si>
     <t>Total</t>
@@ -3965,14 +3968,14 @@
       <c r="C119" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D119" s="5" t="s">
-        <v>204</v>
+      <c r="D119" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>11</v>
+        <v>323</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3980,10 +3983,10 @@
         <v>307</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>204</v>
@@ -3997,13 +4000,13 @@
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
@@ -4012,18 +4015,18 @@
         <v>10</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
@@ -4032,18 +4035,18 @@
         <v>55</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>146</v>
@@ -4052,18 +4055,18 @@
         <v>10</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>204</v>
@@ -4077,13 +4080,13 @@
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>204</v>
@@ -4097,13 +4100,13 @@
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>9</v>
@@ -4112,18 +4115,18 @@
         <v>10</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>9</v>
@@ -4132,18 +4135,18 @@
         <v>10</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>9</v>
@@ -4157,13 +4160,13 @@
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>9</v>
@@ -4177,13 +4180,13 @@
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4197,13 +4200,13 @@
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>9</v>
@@ -4217,13 +4220,13 @@
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>146</v>
@@ -4232,18 +4235,18 @@
         <v>55</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>9</v>
@@ -4257,13 +4260,13 @@
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D134" s="4" t="s">
         <v>146</v>
@@ -4272,18 +4275,18 @@
         <v>55</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>204</v>
@@ -4292,7 +4295,7 @@
         <v>55</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -4313,17 +4316,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4331,10 +4334,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4342,10 +4345,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4356,7 +4359,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4364,26 +4367,26 @@
         <v>204</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B9" s="13">
         <v>134</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4400,7 +4403,7 @@
         <v>204</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4612,13 +4615,13 @@
         <v>307</v>
       </c>
       <c r="B25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25">
         <v>7</v>
@@ -4626,7 +4629,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4643,7 +4646,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Auto-detect frequently-visited spots as favorites
The app now notices when you keep returning to a place and saves it as a
favorite on its own — still entirely on-device.

- lib/location.js: visit clustering (120m radius, distinct visits ≥3h apart),
  monthly pruning; when a cluster reaches 4+ visits in 30 days it's auto-saved
  as a favorite ("A spot you visit often", renameable). New scanLocation()
  does one geolocation read and returns both the nearest favorite (for a nudge)
  and any freshly auto-added spot. Clusters live only in localStorage.
- Chat.jsx: the location effect uses scanLocation; when a spot is auto-saved,
  a companion mentions it ("I've noticed you come here a lot — saved it ✦").

Client-only; no worker change. Build clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="380">
   <si>
     <t>Category</t>
   </si>
@@ -626,7 +626,16 @@
     <t>Companion nudge when near a saved favorite spot</t>
   </si>
   <si>
-    <t>NEW; on-device, lib/location.js favorites + nearbyFavorite</t>
+    <t>NEW; on-device, lib/location.js favorites + scanLocation</t>
+  </si>
+  <si>
+    <t>Auto-detected frequent spots</t>
+  </si>
+  <si>
+    <t>Repeat visits (4+/month) auto-saved as a favorite, on-device</t>
+  </si>
+  <si>
+    <t>NEW; visit clustering in lib/location.js, fully local</t>
   </si>
   <si>
     <t>Preference-aware filtering</t>
@@ -1118,7 +1127,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 134 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 135 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1587,7 +1596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3132,7 +3141,7 @@
         <v>9</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>207</v>
@@ -3140,33 +3149,33 @@
     </row>
     <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="C78" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="D78" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="79" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>9</v>
@@ -3175,12 +3184,12 @@
         <v>10</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>213</v>
+        <v>11</v>
       </c>
     </row>
     <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>214</v>
@@ -3188,11 +3197,11 @@
       <c r="C80" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D80" s="4" t="s">
-        <v>146</v>
+      <c r="D80" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>216</v>
@@ -3200,7 +3209,7 @@
     </row>
     <row r="81" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>217</v>
@@ -3208,11 +3217,11 @@
       <c r="C81" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D81" s="3" t="s">
-        <v>9</v>
+      <c r="D81" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>219</v>
@@ -3220,7 +3229,7 @@
     </row>
     <row r="82" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>220</v>
@@ -3228,39 +3237,39 @@
       <c r="C82" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="83" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="C83" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="D83" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D83" s="4" t="s">
-        <v>146</v>
-      </c>
       <c r="E83" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>226</v>
+        <v>11</v>
       </c>
     </row>
     <row r="84" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>227</v>
@@ -3268,8 +3277,8 @@
       <c r="C84" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D84" s="3" t="s">
-        <v>9</v>
+      <c r="D84" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>10</v>
@@ -3280,7 +3289,7 @@
     </row>
     <row r="85" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>230</v>
@@ -3292,7 +3301,7 @@
         <v>9</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>232</v>
@@ -3300,7 +3309,7 @@
     </row>
     <row r="86" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>233</v>
@@ -3308,11 +3317,11 @@
       <c r="C86" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D86" s="4" t="s">
-        <v>146</v>
+      <c r="D86" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>235</v>
@@ -3320,7 +3329,7 @@
     </row>
     <row r="87" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>236</v>
@@ -3328,11 +3337,11 @@
       <c r="C87" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D87" s="3" t="s">
-        <v>9</v>
+      <c r="D87" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>238</v>
@@ -3340,7 +3349,7 @@
     </row>
     <row r="88" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>239</v>
@@ -3348,8 +3357,8 @@
       <c r="C88" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D88" s="5" t="s">
-        <v>222</v>
+      <c r="D88" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>55</v>
@@ -3360,7 +3369,7 @@
     </row>
     <row r="89" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>242</v>
@@ -3369,10 +3378,10 @@
         <v>243</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>244</v>
@@ -3380,27 +3389,27 @@
     </row>
     <row r="90" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="C90" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="D90" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F90" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="91" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>249</v>
@@ -3412,7 +3421,7 @@
         <v>9</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>251</v>
@@ -3420,7 +3429,7 @@
     </row>
     <row r="92" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>252</v>
@@ -3435,32 +3444,32 @@
         <v>55</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
     </row>
     <row r="93" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>256</v>
+        <v>235</v>
       </c>
     </row>
     <row r="94" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>257</v>
@@ -3480,7 +3489,7 @@
     </row>
     <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>260</v>
@@ -3488,8 +3497,8 @@
       <c r="C95" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D95" s="5" t="s">
-        <v>222</v>
+      <c r="D95" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>10</v>
@@ -3500,33 +3509,33 @@
     </row>
     <row r="96" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="D96" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F96" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="97" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>9</v>
@@ -3540,27 +3549,27 @@
     </row>
     <row r="98" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>270</v>
+        <v>11</v>
       </c>
     </row>
     <row r="99" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>271</v>
@@ -3580,7 +3589,7 @@
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>274</v>
@@ -3592,7 +3601,7 @@
         <v>9</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>276</v>
@@ -3600,7 +3609,7 @@
     </row>
     <row r="101" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>277</v>
@@ -3620,7 +3629,7 @@
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>148</v>
+        <v>266</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>280</v>
@@ -3640,7 +3649,7 @@
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>263</v>
+        <v>148</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>283</v>
@@ -3648,8 +3657,8 @@
       <c r="C103" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D103" s="5" t="s">
-        <v>222</v>
+      <c r="D103" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>118</v>
@@ -3660,7 +3669,7 @@
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>286</v>
@@ -3668,11 +3677,11 @@
       <c r="C104" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D104" s="3" t="s">
-        <v>9</v>
+      <c r="D104" s="5" t="s">
+        <v>225</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>288</v>
@@ -3680,7 +3689,7 @@
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>289</v>
@@ -3692,21 +3701,21 @@
         <v>9</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>11</v>
+        <v>291</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
@@ -3720,33 +3729,33 @@
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>9</v>
@@ -3755,18 +3764,18 @@
         <v>55</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>9</v>
@@ -3775,18 +3784,18 @@
         <v>55</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>52</v>
+        <v>235</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>9</v>
@@ -3800,19 +3809,19 @@
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>52</v>
@@ -3820,36 +3829,36 @@
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>222</v>
+        <v>305</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>118</v>
@@ -3860,7 +3869,7 @@
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>307</v>
+        <v>266</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>308</v>
@@ -3868,19 +3877,19 @@
       <c r="C114" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D114" s="3" t="s">
-        <v>9</v>
+      <c r="D114" s="5" t="s">
+        <v>225</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>310</v>
+        <v>11</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>311</v>
@@ -3892,35 +3901,35 @@
         <v>9</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>232</v>
+        <v>313</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>315</v>
+        <v>235</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>316</v>
@@ -3932,7 +3941,7 @@
         <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>318</v>
@@ -3940,7 +3949,7 @@
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>319</v>
@@ -3952,35 +3961,35 @@
         <v>9</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>232</v>
+        <v>321</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>323</v>
+        <v>235</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>324</v>
@@ -4000,27 +4009,27 @@
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B121" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="C121" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="D121" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F121" s="2" t="s">
         <v>329</v>
-      </c>
-      <c r="D121" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F121" s="2" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>331</v>
@@ -4032,7 +4041,7 @@
         <v>9</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>333</v>
@@ -4040,7 +4049,7 @@
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>334</v>
@@ -4048,11 +4057,11 @@
       <c r="C123" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D123" s="4" t="s">
-        <v>146</v>
+      <c r="D123" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F123" s="2" t="s">
         <v>336</v>
@@ -4060,7 +4069,7 @@
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>337</v>
@@ -4068,28 +4077,28 @@
       <c r="C124" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D124" s="5" t="s">
-        <v>222</v>
+      <c r="D124" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>11</v>
+        <v>339</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>118</v>
@@ -4100,7 +4109,7 @@
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>342</v>
@@ -4108,19 +4117,19 @@
       <c r="C126" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="D126" s="3" t="s">
-        <v>9</v>
+      <c r="D126" s="5" t="s">
+        <v>225</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>344</v>
+        <v>11</v>
       </c>
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>345</v>
@@ -4140,7 +4149,7 @@
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>348</v>
@@ -4155,38 +4164,38 @@
         <v>10</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>52</v>
+        <v>350</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>232</v>
+        <v>52</v>
       </c>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4195,18 +4204,18 @@
         <v>55</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>9</v>
@@ -4215,32 +4224,32 @@
         <v>55</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>52</v>
+        <v>235</v>
       </c>
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="D132" s="4" t="s">
-        <v>146</v>
+        <v>358</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>358</v>
+        <v>52</v>
       </c>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>359</v>
@@ -4248,39 +4257,39 @@
       <c r="C133" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="D133" s="3" t="s">
-        <v>9</v>
+      <c r="D133" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>52</v>
+        <v>361</v>
       </c>
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="D134" s="4" t="s">
-        <v>146</v>
+        <v>363</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>363</v>
+        <v>52</v>
       </c>
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>364</v>
@@ -4288,8 +4297,8 @@
       <c r="C135" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D135" s="5" t="s">
-        <v>222</v>
+      <c r="D135" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>55</v>
@@ -4298,8 +4307,28 @@
         <v>366</v>
       </c>
     </row>
+    <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F135"/>
+  <autoFilter ref="A1:F136"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4316,17 +4345,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4334,10 +4363,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4345,10 +4374,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C6" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4359,34 +4388,34 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B8">
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B9" s="13">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4400,10 +4429,10 @@
         <v>146</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4530,7 +4559,7 @@
         <v>193</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -4539,12 +4568,12 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -4561,7 +4590,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -4578,7 +4607,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B23">
         <v>5</v>
@@ -4595,7 +4624,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B24">
         <v>14</v>
@@ -4612,7 +4641,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B25">
         <v>7</v>
@@ -4629,7 +4658,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -4646,7 +4675,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B27">
         <v>7</v>

</xml_diff>

<commit_message>
Sentience: dreams, closeness milestones, inner-world idle thoughts
- Dreams while sleeping: a sleeping companion dreams (ai.generateDream — short,
  surreal, faintly shaped by their fears/self); on waking they may recount it,
  and the current dream shows on their profile. Generated on open when due.
- Closeness milestones: when the bond crosses up into a new stage (warming →
  close → deeply bonded) the companion marks the moment once with a heartfelt
  line; remembered via stageSeen so it never repeats.
- Inner-world idle thoughts: unprompted lulls now pull from what's actually on
  the companion's mind — their current mood, preoccupation, and stable self —
  instead of generic check-ins.

Unit-tested ranks/dream gating; build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="409">
   <si>
     <t>Category</t>
   </si>
@@ -1181,10 +1181,37 @@
     <t>NEW; ai.generateJournalEntry, ~per visit when due</t>
   </si>
   <si>
+    <t>Dreams while sleeping</t>
+  </si>
+  <si>
+    <t>Sleeping companions dream; may recount on waking; shown on profile</t>
+  </si>
+  <si>
+    <t>NEW; ai.generateDream, dreamDue, recount on wake</t>
+  </si>
+  <si>
+    <t>Closeness milestones</t>
+  </si>
+  <si>
+    <t>Companion marks the moment when a bond deepens a stage, once</t>
+  </si>
+  <si>
+    <t>NEW; stageRank + milestoneLine, stageSeen on companion</t>
+  </si>
+  <si>
+    <t>Inner-world idle thoughts</t>
+  </si>
+  <si>
+    <t>Unprompted thoughts drawn from current mood/preoccupation/self</t>
+  </si>
+  <si>
+    <t>NEW; idle intent + innerLifeBlock in prompt</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 141 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 144 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1656,7 +1683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4507,8 +4534,68 @@
         <v>388</v>
       </c>
     </row>
+    <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F145" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F142"/>
+  <autoFilter ref="A1:F145"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4525,17 +4612,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>389</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>390</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>391</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4543,10 +4630,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4554,10 +4641,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C6" t="s">
-        <v>394</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4568,7 +4655,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4579,23 +4666,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>396</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
       <c r="B9" s="13">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4612,7 +4699,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4705,7 +4792,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -4714,7 +4801,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sentience: temporal memory + inter-companion gossip
- Temporal memory: memory items now carry their "when" into the prompt
  (relativeTime), so companions can say "you mentioned this a few days ago"
  / "last week you were excited about…" instead of floating timeless facts.
- Inter-companion gossip: while companions catch up (ambient on open), they
  trade an impression of the user with each other; the listener absorbs it as
  an "overheard" memory, attributed to the source ("Maya mentioned this about
  you"). Strictly impressions — preferences/traits only, never private facts,
  events, or relationships — so private-chat secrets still never leak. This
  lets a companion come to know something you only told another, the way a
  real friend group works.

6 unit tests (temporal + gossip share/dedupe/attribution); build clean.
Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="427">
   <si>
     <t>Category</t>
   </si>
@@ -1244,10 +1244,28 @@
     <t>NEW; worker innerLine from synced want/journal</t>
   </si>
   <si>
+    <t>Temporal memory</t>
+  </si>
+  <si>
+    <t>Companions reference WHEN things happened (yesterday, last week)</t>
+  </si>
+  <si>
+    <t>NEW; relativeTime in memory block</t>
+  </si>
+  <si>
+    <t>Inter-companion gossip</t>
+  </si>
+  <si>
+    <t>Companions share impressions of you with each other (overheard, attributed)</t>
+  </si>
+  <si>
+    <t>NEW; gossipPick/absorbOverheard, persona-only, never private facts</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 148 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 150 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1719,7 +1737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4710,8 +4728,48 @@
         <v>409</v>
       </c>
     </row>
+    <row r="150" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>415</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F149"/>
+  <autoFilter ref="A1:F151"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4728,17 +4786,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4746,10 +4804,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4757,10 +4815,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4771,7 +4829,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4782,23 +4840,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B9" s="13">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4815,7 +4873,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4908,7 +4966,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -4917,7 +4975,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sentience: peer opinions + mood contagion
- Peer opinions: each companion forms distinct, in-character feelings about the
  others (warmth, friction, admiration, a little jealousy) via ai.generatePeerViews,
  refreshed ~every 5 days. Injected into GROUP prompts (peerViewsBlock) so they
  treat each other like people with history, and shown under each profile's
  Relationships card.
- Mood contagion: the room's collective mood — a blend of every awake
  companion's current inner state (roomMood) — is injected into group prompts,
  so they pick up on and respond to each other's energy, and gently attend to
  whoever seems low.

Both are group-only and read existing per-companion inner state. 5 unit tests;
build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="433">
   <si>
     <t>Category</t>
   </si>
@@ -1262,10 +1262,28 @@
     <t>NEW; gossipPick/absorbOverheard, persona-only, never private facts</t>
   </si>
   <si>
+    <t>Peer opinions</t>
+  </si>
+  <si>
+    <t>Each companion forms distinct feelings about the others; colors group chat + shown on profile</t>
+  </si>
+  <si>
+    <t>NEW; ai.generatePeerViews, peerViewsBlock (group-only)</t>
+  </si>
+  <si>
+    <t>Mood contagion</t>
+  </si>
+  <si>
+    <t>The room's collective mood (each companion's state) shapes the group vibe</t>
+  </si>
+  <si>
+    <t>NEW; roomMood injected into group prompt</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 150 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 152 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1737,7 +1755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4768,8 +4786,48 @@
         <v>415</v>
       </c>
     </row>
+    <row r="152" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F151"/>
+  <autoFilter ref="A1:F153"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4786,17 +4844,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4804,10 +4862,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4815,10 +4873,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4829,7 +4887,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4840,23 +4898,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="B9" s="13">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4873,7 +4931,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4966,7 +5024,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -4975,7 +5033,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sentience: group conflict/sides + shared-history lore
- Group conflict & taking sides: the group-chat prompt now invites companions
  to form alliances, back up whoever they're close to, gang up playfully, and
  spar with whoever they butt heads with — affectionate banter and mild
  conflict instead of forced consensus (works with the peer-opinions layer).
- Shared history ("lore"): the group distills memorable moments they've been
  through together into short "remember when…" lines (ai.generateSharedMoment,
  ~daily when there's been enough chat). Stored at session level (persists +
  syncs), injected into prompts (loreBlock) so any companion can reference them,
  and surfaced as "your story together" at the bottom of the Space.

7 unit tests for lore cadence/cap/block; build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="439">
   <si>
     <t>Category</t>
   </si>
@@ -1280,10 +1280,28 @@
     <t>NEW; roomMood injected into group prompt</t>
   </si>
   <si>
+    <t>Group conflict &amp; sides</t>
+  </si>
+  <si>
+    <t>Companions form alliances, take sides, playfully spar in group chat</t>
+  </si>
+  <si>
+    <t>NEW; group MODE guidance + peer opinions</t>
+  </si>
+  <si>
+    <t>Shared history timeline</t>
+  </si>
+  <si>
+    <t>Group distills memorable moments into lore they reference (remember when)</t>
+  </si>
+  <si>
+    <t>NEW; ai.generateSharedMoment, loreBlock, shown in Space</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 152 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 154 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1301,7 +1319,7 @@
     <t>5%</t>
   </si>
   <si>
-    <t>7%</t>
+    <t>6%</t>
   </si>
   <si>
     <t>Total</t>
@@ -1755,7 +1773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F153"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4826,8 +4844,48 @@
         <v>421</v>
       </c>
     </row>
+    <row r="154" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F153"/>
+  <autoFilter ref="A1:F155"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4844,17 +4902,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4862,10 +4920,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4873,10 +4931,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4887,7 +4945,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4898,23 +4956,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="B9" s="13">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4931,7 +4989,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5007,7 +5065,7 @@
         <v>105</v>
       </c>
       <c r="B17">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -5016,7 +5074,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5024,7 +5082,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -5033,7 +5091,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sentience: walk-in scenes + rupture & repair
- Walk into a scene: ~half the time on open, the ambient exchange is framed as
  in-progress — you arrive mid-conversation and a companion notices/greets you
  in the last line (ambientThreadAI arriving mode; "you walk in on them…"
  divider).
- Rupture & repair: a long silence (3+ weeks) leaves a once-close companion in
  the "distant" stage — on return they're hurt and guarded (a one-time rift
  line); sustained re-engagement heals it and triggers a reconciliation moment.
  Tracked with riftSeen/repairSeen so the arc can cycle without repeating.

Build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="445">
   <si>
     <t>Category</t>
   </si>
@@ -1298,10 +1298,28 @@
     <t>NEW; ai.generateSharedMoment, loreBlock, shown in Space</t>
   </si>
   <si>
+    <t>Walk into a scene</t>
+  </si>
+  <si>
+    <t>Sometimes you arrive mid-conversation and a companion notices you</t>
+  </si>
+  <si>
+    <t>NEW; ambientThreadAI arriving mode + walk-in divider</t>
+  </si>
+  <si>
+    <t>Rupture &amp; repair</t>
+  </si>
+  <si>
+    <t>Long neglect leaves a once-close companion hurt/guarded; re-engagement heals with a reconciliation moment</t>
+  </si>
+  <si>
+    <t>NEW; distant stage + riftSeen/repairSeen arc</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 154 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 156 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1316,7 +1334,7 @@
     <t>89%</t>
   </si>
   <si>
-    <t>5%</t>
+    <t>4%</t>
   </si>
   <si>
     <t>6%</t>
@@ -1773,7 +1791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4884,8 +4902,48 @@
         <v>427</v>
       </c>
     </row>
+    <row r="156" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F156" s="2" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F157" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F155"/>
+  <autoFilter ref="A1:F157"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4902,17 +4960,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4920,10 +4978,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4931,10 +4989,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C6" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4945,7 +5003,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4956,23 +5014,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B9" s="13">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4989,7 +5047,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5065,7 +5123,7 @@
         <v>105</v>
       </c>
       <c r="B17">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -5074,7 +5132,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5082,7 +5140,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -5091,7 +5149,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sentience: occasion awareness (dates, holidays, birthday, anniversary)
Grounds companions in real time so they're aware of the world's calendar and
the relationship's milestones.

- lib/occasion.js: occasionContext() injects today's weekday/date, season,
  time of day, and any holiday (fixed + US Thanksgiving) into every prompt, plus
  flags the user's birthday (today/soon) from their DOB; birthdayStatus() and
  monthsKnown() helpers.
- Chat: a companion wishes the user happy birthday (once per year, localStorage-
  guarded) and marks each monthly anniversary of when you met once ("it's been
  3 months since we met…", a special line at 1 year). Anniversary uses the
  bornAt seeded by the growth system.

Companions reference the day/season/occasion only when it fits. 9 unit tests;
build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="451">
   <si>
     <t>Category</t>
   </si>
@@ -1325,10 +1325,19 @@
     <t>NEW; ai.generateGrowth ~monthly, knownDuration, growth log</t>
   </si>
   <si>
+    <t>Occasion awareness</t>
+  </si>
+  <si>
+    <t>Companions know the date/season/holidays + the user's birthday and anniversary; celebrate them</t>
+  </si>
+  <si>
+    <t>NEW; lib/occasion.js context + birthday/anniversary greetings</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 157 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 158 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1800,7 +1809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4971,8 +4980,28 @@
         <v>436</v>
       </c>
     </row>
+    <row r="159" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F158"/>
+  <autoFilter ref="A1:F159"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4989,17 +5018,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5007,10 +5036,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5018,10 +5047,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5032,7 +5061,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5043,23 +5072,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B9" s="13">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5076,7 +5105,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5169,7 +5198,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -5178,7 +5207,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Inner-life generation budget + mood-reactive avatars
- Safeguard: the on-open inner-life effect now caps total AI generations at 3
  per open, in priority order (self > journal > dream > want > shift > peer
  views > shared moment > growth). Anything skipped stays "due" and runs on a
  later open, so a fresh account never fires a burst of calls at once.
- Mood-reactive avatars: vitality() maps a companion's current inner state to a
  0-1 liveliness; the Avatar's glow and star brightness scale with it (and
  slightly desaturate when low), and in the Space lower-energy companions drift
  more slowly. Sleeping reads as dim. Pure client, no AI — a quiet visual
  sentience cue.

Tests for vitality; build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="458">
   <si>
     <t>Category</t>
   </si>
@@ -1334,10 +1334,31 @@
     <t>NEW; lib/occasion.js context + birthday/anniversary greetings</t>
   </si>
   <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Inner-life generation budget</t>
+  </si>
+  <si>
+    <t>Caps inner-life AI generations per open (max 3); rest run next open</t>
+  </si>
+  <si>
+    <t>NEW; prioritized, prevents first-open AI burst</t>
+  </si>
+  <si>
+    <t>Mood-reactive avatars</t>
+  </si>
+  <si>
+    <t>Avatar brightness/liveliness reflects the companion's current inner state</t>
+  </si>
+  <si>
+    <t>NEW; vitality() -&gt; Avatar glow/stars + Space float speed</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 158 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 160 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1809,7 +1830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F159"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5000,8 +5021,48 @@
         <v>439</v>
       </c>
     </row>
+    <row r="160" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F161" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F159"/>
+  <autoFilter ref="A1:F161"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5009,7 +5070,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -5018,17 +5079,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5036,10 +5097,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5047,10 +5108,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C6" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5061,7 +5122,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5072,23 +5133,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B9" s="13">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5105,7 +5166,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5300,7 +5361,7 @@
         <v>267</v>
       </c>
       <c r="B24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -5309,7 +5370,7 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5361,6 +5422,23 @@
       </c>
       <c r="E27">
         <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>440</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sentience: inside jokes + identity-curiosity questions
- Inside jokes: the group coins a running bit from recent chat
  (ai.generateInsideJoke, budgeted, ~every 2 days) and calls back to it later;
  injected via jokesBlock, persisted + synced like lore.
- Identity curiosity: now and then (low probability, once per session, after a
  delay) a companion asks the user something about who they are or how they're
  seen ("do you think I've changed since we met?"), pulling them into reflecting
  on the companion as a person.

7 unit tests; build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="464">
   <si>
     <t>Category</t>
   </si>
@@ -1355,10 +1355,28 @@
     <t>NEW; vitality() -&gt; Avatar glow/stars + Space float speed</t>
   </si>
   <si>
+    <t>Inside jokes</t>
+  </si>
+  <si>
+    <t>Group coins running bits and calls back to them later</t>
+  </si>
+  <si>
+    <t>NEW; ai.generateInsideJoke, jokesBlock, budgeted</t>
+  </si>
+  <si>
+    <t>Identity curiosity</t>
+  </si>
+  <si>
+    <t>Companions occasionally ask the user about who they are / how they're seen</t>
+  </si>
+  <si>
+    <t>NEW; identityQuestion, low-probability once/session</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 160 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 162 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1370,7 +1388,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>89%</t>
+    <t>90%</t>
   </si>
   <si>
     <t>4%</t>
@@ -1830,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5061,8 +5079,48 @@
         <v>446</v>
       </c>
     </row>
+    <row r="162" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F161"/>
+  <autoFilter ref="A1:F163"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5079,17 +5137,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5097,10 +5155,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5108,10 +5166,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C6" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5122,7 +5180,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5133,23 +5191,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B9" s="13">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5166,7 +5224,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5259,7 +5317,7 @@
         <v>148</v>
       </c>
       <c r="B18">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -5268,7 +5326,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add "Your story so far" keepsake panel + note smoke test
- StorySoFar.jsx (chat menu → 📖): collects the relationship's accumulated
  artifacts in one place — shared history ("remember when…"), inside jokes, and
  letters from each companion — making the inner-life system tangible.
- Verified via a Playwright load test of the production build that the app boots
  Welcome → onboarding and a seeded session lands in Chat (all inner-life
  effects) with no runtime/React errors.

Build clean. Client-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="494">
   <si>
     <t>Category</t>
   </si>
@@ -1445,10 +1445,28 @@
     <t>NEW; lib/location.weatherNow, cached, coarse coords</t>
   </si>
   <si>
+    <t>Story so far panel</t>
+  </si>
+  <si>
+    <t>Keepsake view of shared history, inside jokes, and letters</t>
+  </si>
+  <si>
+    <t>NEW; screens/StorySoFar.jsx, chat menu</t>
+  </si>
+  <si>
+    <t>Runtime smoke test</t>
+  </si>
+  <si>
+    <t>Verified app boots Welcome-&gt;onboarding-&gt;Chat with no runtime errors</t>
+  </si>
+  <si>
+    <t>Playwright load test of production build</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 170 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 172 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1920,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5351,8 +5369,48 @@
         <v>476</v>
       </c>
     </row>
+    <row r="172" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F172" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="D173" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F173" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F171"/>
+  <autoFilter ref="A1:F173"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5369,17 +5427,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5387,10 +5445,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5398,10 +5456,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C6" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5412,7 +5470,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5423,23 +5481,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B9" s="13">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5456,7 +5514,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5651,7 +5709,7 @@
         <v>267</v>
       </c>
       <c r="B24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -5660,7 +5718,7 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5719,7 +5777,7 @@
         <v>440</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -5728,7 +5786,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish: one companion-initiated beat per open (anti-flood coordinator)
Opening the app could stack several unprompted "beats" at once (milestone +
vulnerability + rupture/repair + birthday/anniversary + curiosity). Added a
shared claimBeat() gate (3-minute cooldown) that all of these check right
before posting; the first eligible one fires, the rest defer and retry later —
so a return never floods the chat. Verified via browser smoke test (exactly one
beat fired, no runtime errors).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="497">
   <si>
     <t>Category</t>
   </si>
@@ -1463,10 +1463,19 @@
     <t>Playwright load test of production build</t>
   </si>
   <si>
+    <t>Beat coordinator (polish)</t>
+  </si>
+  <si>
+    <t>At most one companion-initiated emotional beat per open (3-min cooldown)</t>
+  </si>
+  <si>
+    <t>NEW; claimBeat() gates milestone/vulnerability/rift/occasion/curiosity</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 172 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 173 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1938,7 +1947,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5409,8 +5418,28 @@
         <v>482</v>
       </c>
     </row>
+    <row r="174" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="D174" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F173"/>
+  <autoFilter ref="A1:F174"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5427,17 +5456,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5445,10 +5474,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5456,10 +5485,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C6" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5470,7 +5499,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5481,23 +5510,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B9" s="13">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5514,7 +5543,7 @@
         <v>226</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5777,7 +5806,7 @@
         <v>440</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -5786,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Defer lounge decoration to a later-stage customization
Per owner direction, lounge/Space decoration is intentionally planned
for months out, not the near-term queue. Drop it to P3 and note the
deferral in the tracker; regenerate the xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="499">
   <si>
     <t>Category</t>
   </si>
@@ -884,7 +884,10 @@
     <t>Customize the Space: background pictures, tiles, patterns/themes</t>
   </si>
   <si>
-    <t>User request; decorate the sitting space (uploads or preset patterns)</t>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>User request; intentionally deferred months out as a later-stage customization (uploads or preset patterns)</t>
   </si>
   <si>
     <t>Cosmetic customization</t>
@@ -4035,10 +4038,10 @@
         <v>227</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>118</v>
+        <v>290</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4046,10 +4049,10 @@
         <v>268</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
@@ -4058,7 +4061,7 @@
         <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4066,10 +4069,10 @@
         <v>268</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
@@ -4086,10 +4089,10 @@
         <v>268</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
@@ -4106,10 +4109,10 @@
         <v>268</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>9</v>
@@ -4126,10 +4129,10 @@
         <v>268</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>9</v>
@@ -4146,10 +4149,10 @@
         <v>268</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>9</v>
@@ -4166,10 +4169,10 @@
         <v>268</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>9</v>
@@ -4186,10 +4189,10 @@
         <v>268</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>9</v>
@@ -4206,10 +4209,10 @@
         <v>268</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>227</v>
@@ -4226,10 +4229,10 @@
         <v>268</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>227</v>
@@ -4243,13 +4246,13 @@
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>9</v>
@@ -4258,18 +4261,18 @@
         <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>9</v>
@@ -4283,13 +4286,13 @@
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>9</v>
@@ -4298,18 +4301,18 @@
         <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>9</v>
@@ -4318,18 +4321,18 @@
         <v>118</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>9</v>
@@ -4343,13 +4346,13 @@
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>9</v>
@@ -4358,18 +4361,18 @@
         <v>118</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
@@ -4378,18 +4381,18 @@
         <v>118</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
@@ -4398,18 +4401,18 @@
         <v>10</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>9</v>
@@ -4418,18 +4421,18 @@
         <v>55</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>147</v>
@@ -4438,18 +4441,18 @@
         <v>10</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>227</v>
@@ -4463,13 +4466,13 @@
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>227</v>
@@ -4483,13 +4486,13 @@
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>9</v>
@@ -4498,18 +4501,18 @@
         <v>10</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>9</v>
@@ -4518,18 +4521,18 @@
         <v>10</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>9</v>
@@ -4543,13 +4546,13 @@
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4563,13 +4566,13 @@
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>9</v>
@@ -4583,13 +4586,13 @@
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>9</v>
@@ -4603,13 +4606,13 @@
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>147</v>
@@ -4618,18 +4621,18 @@
         <v>55</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>9</v>
@@ -4643,13 +4646,13 @@
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>147</v>
@@ -4658,18 +4661,18 @@
         <v>55</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>227</v>
@@ -4678,7 +4681,7 @@
         <v>55</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="137" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4686,10 +4689,10 @@
         <v>105</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>9</v>
@@ -4698,7 +4701,7 @@
         <v>55</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="138" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4706,10 +4709,10 @@
         <v>105</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>9</v>
@@ -4718,7 +4721,7 @@
         <v>118</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4726,10 +4729,10 @@
         <v>149</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>9</v>
@@ -4738,7 +4741,7 @@
         <v>55</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="140" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4746,10 +4749,10 @@
         <v>149</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>9</v>
@@ -4758,7 +4761,7 @@
         <v>55</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="141" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4766,10 +4769,10 @@
         <v>149</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>9</v>
@@ -4778,7 +4781,7 @@
         <v>55</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="142" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4786,10 +4789,10 @@
         <v>149</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>9</v>
@@ -4798,7 +4801,7 @@
         <v>118</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4806,10 +4809,10 @@
         <v>149</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>9</v>
@@ -4818,7 +4821,7 @@
         <v>118</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4826,10 +4829,10 @@
         <v>149</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>9</v>
@@ -4838,7 +4841,7 @@
         <v>118</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="145" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4846,10 +4849,10 @@
         <v>149</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>9</v>
@@ -4858,7 +4861,7 @@
         <v>118</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="146" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4866,10 +4869,10 @@
         <v>149</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>9</v>
@@ -4878,7 +4881,7 @@
         <v>118</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="147" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4886,10 +4889,10 @@
         <v>149</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>9</v>
@@ -4898,7 +4901,7 @@
         <v>118</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="148" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4906,10 +4909,10 @@
         <v>149</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>9</v>
@@ -4918,18 +4921,18 @@
         <v>118</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="149" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D149" s="3" t="s">
         <v>9</v>
@@ -4938,7 +4941,7 @@
         <v>118</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="150" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4946,10 +4949,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>9</v>
@@ -4958,7 +4961,7 @@
         <v>118</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="151" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4966,10 +4969,10 @@
         <v>149</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D151" s="3" t="s">
         <v>9</v>
@@ -4978,7 +4981,7 @@
         <v>118</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="152" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4986,10 +4989,10 @@
         <v>149</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>9</v>
@@ -4998,7 +5001,7 @@
         <v>118</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="153" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5006,10 +5009,10 @@
         <v>149</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>9</v>
@@ -5018,7 +5021,7 @@
         <v>118</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="154" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5026,10 +5029,10 @@
         <v>105</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>9</v>
@@ -5038,7 +5041,7 @@
         <v>118</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="155" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5046,10 +5049,10 @@
         <v>149</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D155" s="3" t="s">
         <v>9</v>
@@ -5058,7 +5061,7 @@
         <v>118</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="156" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5066,10 +5069,10 @@
         <v>105</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>9</v>
@@ -5078,7 +5081,7 @@
         <v>118</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="157" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5086,10 +5089,10 @@
         <v>149</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>9</v>
@@ -5098,7 +5101,7 @@
         <v>118</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="158" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5106,10 +5109,10 @@
         <v>149</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>9</v>
@@ -5118,7 +5121,7 @@
         <v>55</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="159" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5126,10 +5129,10 @@
         <v>149</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>9</v>
@@ -5138,18 +5141,18 @@
         <v>118</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="160" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>9</v>
@@ -5158,7 +5161,7 @@
         <v>55</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="161" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5166,10 +5169,10 @@
         <v>268</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>9</v>
@@ -5178,7 +5181,7 @@
         <v>118</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="162" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5186,10 +5189,10 @@
         <v>149</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>9</v>
@@ -5198,7 +5201,7 @@
         <v>118</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="163" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5206,10 +5209,10 @@
         <v>149</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>9</v>
@@ -5218,7 +5221,7 @@
         <v>118</v>
       </c>
       <c r="F163" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="164" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5226,10 +5229,10 @@
         <v>149</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>9</v>
@@ -5238,7 +5241,7 @@
         <v>118</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="165" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5246,10 +5249,10 @@
         <v>149</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>9</v>
@@ -5258,7 +5261,7 @@
         <v>118</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="166" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5266,10 +5269,10 @@
         <v>149</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>9</v>
@@ -5278,7 +5281,7 @@
         <v>118</v>
       </c>
       <c r="F166" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="167" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5286,10 +5289,10 @@
         <v>149</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>9</v>
@@ -5298,7 +5301,7 @@
         <v>118</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="168" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5306,10 +5309,10 @@
         <v>149</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>9</v>
@@ -5318,7 +5321,7 @@
         <v>118</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="169" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5326,10 +5329,10 @@
         <v>149</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>9</v>
@@ -5338,7 +5341,7 @@
         <v>118</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="170" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5346,10 +5349,10 @@
         <v>268</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D170" s="3" t="s">
         <v>9</v>
@@ -5358,7 +5361,7 @@
         <v>118</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="171" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5366,10 +5369,10 @@
         <v>194</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D171" s="3" t="s">
         <v>9</v>
@@ -5378,7 +5381,7 @@
         <v>118</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="172" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5386,10 +5389,10 @@
         <v>268</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D172" s="3" t="s">
         <v>9</v>
@@ -5398,18 +5401,18 @@
         <v>118</v>
       </c>
       <c r="F172" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="173" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D173" s="3" t="s">
         <v>9</v>
@@ -5418,18 +5421,18 @@
         <v>55</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="174" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D174" s="3" t="s">
         <v>9</v>
@@ -5438,7 +5441,7 @@
         <v>55</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
   </sheetData>
@@ -5459,17 +5462,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5477,10 +5480,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5491,7 +5494,7 @@
         <v>157</v>
       </c>
       <c r="C6" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5502,7 +5505,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5513,23 +5516,23 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B9" s="13">
         <v>173</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5546,7 +5549,7 @@
         <v>227</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5755,7 +5758,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B25">
         <v>8</v>
@@ -5772,7 +5775,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -5789,7 +5792,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B27">
         <v>7</v>
@@ -5806,7 +5809,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B28">
         <v>3</v>

</xml_diff>

<commit_message>
Make the constellation sigil optional per companion
Add a "Constellation sigil" toggle to the companion editor's Appearance
card. When off, the stars (and the avatar's orbital ring) are hidden,
leaving a clean colour orb / gel blob.

- Persisted as comp.showSigil (default on; syncs with the roster).
- Honoured everywhere the companion is drawn: SquishyBlob (profile
  playground, Appearance preview, The Space) and the inline Avatar
  (chat bubbles, headers) read the flag straight off the companion, so
  no call sites needed changes.

Verified in a real browser: toggling off removes the star circles
(12 -> 0) and back on restores them; no runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -902,10 +902,10 @@
     <t>Cosmetic customization</t>
   </si>
   <si>
-    <t>Recolor a companion: 8-color palette + custom color wheel</t>
-  </si>
-  <si>
-    <t>UPDATED; ToS 4.1; &lt;input type=color&gt; any color</t>
+    <t>Recolor a companion: 8-color palette + custom color wheel; squishiness slider; optional constellation sigil toggle</t>
+  </si>
+  <si>
+    <t>UPDATED; ToS 4.1; &lt;input type=color&gt; any color; comp.blob, comp.showSigil</t>
   </si>
   <si>
     <t>Animated waking sequence</t>

</xml_diff>

<commit_message>
Keep chat pinned to the latest message while typing
New messages no longer hide under the input box. When you're already at
the bottom, the view now stays pinned as the textarea grows with a
multi-line draft and as the on-screen keyboard opens/closes:

- textarea onChange/onFocus call an instant pinBottom() when at-bottom
- a visualViewport resize listener re-pins on keyboard show/hide
- all pinning is gated on a live atBottomRef, so scrolling up to read
  history is never yanked back down

Verified in a real browser: typing a 6-line draft keeps the latest
message in view (distance from bottom stays 0); no runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="507">
   <si>
     <t>Category</t>
   </si>
@@ -953,7 +953,10 @@
     <t>Chat quality-of-life</t>
   </si>
   <si>
-    <t>Timestamps, copy, scroll-to-bottom, multiline</t>
+    <t>Timestamps, copy, scroll-to-bottom, multiline, sticky-to-bottom while typing (input growth + keyboard never hide new messages)</t>
+  </si>
+  <si>
+    <t>UPDATED; pinBottom on input grow/focus + visualViewport resize, gated on at-bottom</t>
   </si>
   <si>
     <t>Offline awareness</t>
@@ -4242,7 +4245,7 @@
         <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>52</v>
+        <v>314</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4250,10 +4253,10 @@
         <v>272</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>9</v>
@@ -4270,10 +4273,10 @@
         <v>272</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>231</v>
@@ -4290,10 +4293,10 @@
         <v>272</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>231</v>
@@ -4307,13 +4310,13 @@
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>9</v>
@@ -4322,18 +4325,18 @@
         <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>9</v>
@@ -4347,13 +4350,13 @@
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>9</v>
@@ -4362,18 +4365,18 @@
         <v>55</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>9</v>
@@ -4382,18 +4385,18 @@
         <v>122</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
@@ -4407,13 +4410,13 @@
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
@@ -4422,18 +4425,18 @@
         <v>122</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>9</v>
@@ -4442,18 +4445,18 @@
         <v>122</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>9</v>
@@ -4462,18 +4465,18 @@
         <v>10</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>9</v>
@@ -4482,18 +4485,18 @@
         <v>55</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>151</v>
@@ -4502,18 +4505,18 @@
         <v>10</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>231</v>
@@ -4527,13 +4530,13 @@
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>231</v>
@@ -4547,13 +4550,13 @@
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>9</v>
@@ -4562,18 +4565,18 @@
         <v>10</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>9</v>
@@ -4582,18 +4585,18 @@
         <v>10</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>9</v>
@@ -4607,13 +4610,13 @@
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>9</v>
@@ -4627,13 +4630,13 @@
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>9</v>
@@ -4647,13 +4650,13 @@
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>9</v>
@@ -4667,13 +4670,13 @@
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>151</v>
@@ -4682,18 +4685,18 @@
         <v>55</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>9</v>
@@ -4707,13 +4710,13 @@
     </row>
     <row r="137" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>151</v>
@@ -4722,18 +4725,18 @@
         <v>55</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="138" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>231</v>
@@ -4742,7 +4745,7 @@
         <v>55</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4750,10 +4753,10 @@
         <v>109</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>9</v>
@@ -4762,7 +4765,7 @@
         <v>55</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="140" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4770,10 +4773,10 @@
         <v>109</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>9</v>
@@ -4782,7 +4785,7 @@
         <v>122</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="141" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4790,10 +4793,10 @@
         <v>153</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>9</v>
@@ -4802,7 +4805,7 @@
         <v>55</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="142" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4810,10 +4813,10 @@
         <v>153</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>9</v>
@@ -4822,7 +4825,7 @@
         <v>55</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4830,10 +4833,10 @@
         <v>153</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>9</v>
@@ -4842,7 +4845,7 @@
         <v>55</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4850,10 +4853,10 @@
         <v>153</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>9</v>
@@ -4862,7 +4865,7 @@
         <v>122</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="145" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4870,10 +4873,10 @@
         <v>153</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>9</v>
@@ -4882,7 +4885,7 @@
         <v>122</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="146" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4890,10 +4893,10 @@
         <v>153</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>9</v>
@@ -4902,7 +4905,7 @@
         <v>122</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="147" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4910,10 +4913,10 @@
         <v>153</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>9</v>
@@ -4922,7 +4925,7 @@
         <v>122</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="148" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4930,10 +4933,10 @@
         <v>153</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>9</v>
@@ -4942,7 +4945,7 @@
         <v>122</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="149" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4950,10 +4953,10 @@
         <v>153</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D149" s="3" t="s">
         <v>9</v>
@@ -4962,7 +4965,7 @@
         <v>122</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="150" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4970,10 +4973,10 @@
         <v>153</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>9</v>
@@ -4982,18 +4985,18 @@
         <v>122</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="151" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D151" s="3" t="s">
         <v>9</v>
@@ -5002,7 +5005,7 @@
         <v>122</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="152" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5010,10 +5013,10 @@
         <v>153</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>9</v>
@@ -5022,7 +5025,7 @@
         <v>122</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="153" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5030,10 +5033,10 @@
         <v>153</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>9</v>
@@ -5042,7 +5045,7 @@
         <v>122</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="154" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5050,10 +5053,10 @@
         <v>153</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>9</v>
@@ -5062,7 +5065,7 @@
         <v>122</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="155" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5070,10 +5073,10 @@
         <v>153</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D155" s="3" t="s">
         <v>9</v>
@@ -5082,7 +5085,7 @@
         <v>122</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="156" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5090,10 +5093,10 @@
         <v>109</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>9</v>
@@ -5102,7 +5105,7 @@
         <v>122</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="157" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5110,10 +5113,10 @@
         <v>153</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>9</v>
@@ -5122,7 +5125,7 @@
         <v>122</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="158" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5130,10 +5133,10 @@
         <v>109</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>9</v>
@@ -5142,7 +5145,7 @@
         <v>122</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="159" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5150,10 +5153,10 @@
         <v>153</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>9</v>
@@ -5162,7 +5165,7 @@
         <v>122</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="160" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5170,10 +5173,10 @@
         <v>153</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>9</v>
@@ -5182,7 +5185,7 @@
         <v>55</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="161" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5190,10 +5193,10 @@
         <v>153</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>9</v>
@@ -5202,18 +5205,18 @@
         <v>122</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="162" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>9</v>
@@ -5222,7 +5225,7 @@
         <v>55</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="163" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5230,10 +5233,10 @@
         <v>272</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>9</v>
@@ -5242,7 +5245,7 @@
         <v>122</v>
       </c>
       <c r="F163" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="164" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5250,10 +5253,10 @@
         <v>153</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>9</v>
@@ -5262,7 +5265,7 @@
         <v>122</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="165" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5270,10 +5273,10 @@
         <v>153</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>9</v>
@@ -5282,7 +5285,7 @@
         <v>122</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="166" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5290,10 +5293,10 @@
         <v>153</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>9</v>
@@ -5302,7 +5305,7 @@
         <v>122</v>
       </c>
       <c r="F166" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="167" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5310,10 +5313,10 @@
         <v>153</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>9</v>
@@ -5322,7 +5325,7 @@
         <v>122</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="168" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5330,10 +5333,10 @@
         <v>153</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>9</v>
@@ -5342,7 +5345,7 @@
         <v>122</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="169" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5350,10 +5353,10 @@
         <v>153</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>9</v>
@@ -5362,7 +5365,7 @@
         <v>122</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="170" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5370,10 +5373,10 @@
         <v>153</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D170" s="3" t="s">
         <v>9</v>
@@ -5382,7 +5385,7 @@
         <v>122</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="171" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5390,10 +5393,10 @@
         <v>153</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D171" s="3" t="s">
         <v>9</v>
@@ -5402,7 +5405,7 @@
         <v>122</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="172" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5410,10 +5413,10 @@
         <v>272</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D172" s="3" t="s">
         <v>9</v>
@@ -5422,7 +5425,7 @@
         <v>122</v>
       </c>
       <c r="F172" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="173" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5430,10 +5433,10 @@
         <v>198</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D173" s="3" t="s">
         <v>9</v>
@@ -5442,7 +5445,7 @@
         <v>122</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="174" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5450,10 +5453,10 @@
         <v>272</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D174" s="3" t="s">
         <v>9</v>
@@ -5462,18 +5465,18 @@
         <v>122</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="175" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D175" s="3" t="s">
         <v>9</v>
@@ -5482,18 +5485,18 @@
         <v>55</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="176" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D176" s="3" t="s">
         <v>9</v>
@@ -5502,7 +5505,7 @@
         <v>55</v>
       </c>
       <c r="F176" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -5523,17 +5526,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5541,10 +5544,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5555,7 +5558,7 @@
         <v>159</v>
       </c>
       <c r="C6" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5566,7 +5569,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5577,23 +5580,23 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B9" s="13">
         <v>175</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5610,7 +5613,7 @@
         <v>231</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5819,7 +5822,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B25">
         <v>8</v>
@@ -5836,7 +5839,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -5853,7 +5856,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B27">
         <v>7</v>
@@ -5870,7 +5873,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B28">
         <v>3</v>

</xml_diff>

<commit_message>
Close SB 243 gaps: crisis-safety page + minor break reminder
California SB 243 (effective Jan 1, 2026) compliance for companion
chatbots:

- Published "Crisis Resources & Safety" page (data/legal.js) documenting
  our crisis-prevention protocol — detection, the resource card, 988 /
  Crisis Text Line / Find a Helpline, limitations, and minor protections.
  Linked from Settings → Legal and from the in-chat crisis card.
- Minor-only "take a break" reminder: for under-18 users, an in-chat note
  every 3 hours of continuous use reminding them companions are AI and to
  take a break (disclosure.breakReminderDue + a gated Chat effect).

Verified in a real browser (seeded under-18 session): the break reminder
fires once the 3h clock elapses, and the Safety page renders with the
protocol details and 988; no runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="523">
   <si>
     <t>Category</t>
   </si>
@@ -599,6 +599,18 @@
     <t>UPDATED Partial-&gt;Built; lib/crisis.js</t>
   </si>
   <si>
+    <t>Compliance</t>
+  </si>
+  <si>
+    <t>SB 243 companion-chatbot safeguards</t>
+  </si>
+  <si>
+    <t>California SB 243 gaps closed: published Crisis Resources &amp; Safety page (crisis-prevention protocol + 988/741741) linked from Settings + crisis card, and a minor-only 'take a break' reminder every 3 hours of continuous use (with AI-not-human reminder)</t>
+  </si>
+  <si>
+    <t>NEW; data/legal.js safety doc, disclosure.breakReminderDue, Chat minor effect</t>
+  </si>
+  <si>
     <t>Therapist suggestions</t>
   </si>
   <si>
@@ -1541,7 +1553,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 179 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 180 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -2013,7 +2025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F180"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3466,22 +3478,22 @@
     </row>
     <row r="73" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="74" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3489,10 +3501,10 @@
         <v>181</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>9</v>
@@ -3501,12 +3513,12 @@
         <v>55</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="75" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>201</v>
+        <v>181</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>202</v>
@@ -3526,13 +3538,13 @@
     </row>
     <row r="76" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>9</v>
@@ -3541,18 +3553,18 @@
         <v>55</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="77" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>9</v>
@@ -3561,38 +3573,38 @@
         <v>55</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="79" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>9</v>
@@ -3601,32 +3613,32 @@
         <v>122</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="81" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>221</v>
@@ -3638,21 +3650,21 @@
         <v>9</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>11</v>
+        <v>223</v>
       </c>
     </row>
     <row r="82" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>9</v>
@@ -3661,72 +3673,72 @@
         <v>10</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>225</v>
+        <v>11</v>
       </c>
     </row>
     <row r="83" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D83" s="4" t="s">
-        <v>151</v>
+        <v>228</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="84" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>9</v>
+        <v>231</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="85" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D85" s="5" t="s">
         <v>234</v>
       </c>
+      <c r="D85" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E85" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>11</v>
+        <v>235</v>
       </c>
     </row>
     <row r="86" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>236</v>
@@ -3734,139 +3746,139 @@
       <c r="C86" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D86" s="4" t="s">
-        <v>151</v>
+      <c r="D86" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>238</v>
+        <v>11</v>
       </c>
     </row>
     <row r="87" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>9</v>
+        <v>241</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="88" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="89" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="D89" s="4" t="s">
-        <v>151</v>
+        <v>247</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="90" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>9</v>
+        <v>250</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="91" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="D91" s="5" t="s">
-        <v>234</v>
+        <v>253</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="92" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="93" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>258</v>
@@ -3874,8 +3886,8 @@
       <c r="C93" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D93" s="3" t="s">
-        <v>9</v>
+      <c r="D93" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>10</v>
@@ -3886,33 +3898,33 @@
     </row>
     <row r="94" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>9</v>
@@ -3921,18 +3933,18 @@
         <v>55</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="96" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>9</v>
@@ -3941,38 +3953,38 @@
         <v>55</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
     </row>
     <row r="97" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>271</v>
+        <v>248</v>
       </c>
     </row>
     <row r="98" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>9</v>
@@ -3981,18 +3993,18 @@
         <v>10</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>9</v>
@@ -4001,12 +4013,12 @@
         <v>10</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>279</v>
@@ -4021,18 +4033,18 @@
         <v>10</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>11</v>
+        <v>281</v>
       </c>
     </row>
     <row r="101" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>9</v>
@@ -4046,33 +4058,33 @@
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>285</v>
+        <v>11</v>
       </c>
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>9</v>
@@ -4081,18 +4093,18 @@
         <v>55</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>9</v>
@@ -4101,38 +4113,38 @@
         <v>55</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>9</v>
@@ -4141,18 +4153,18 @@
         <v>122</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>153</v>
+        <v>282</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>9</v>
@@ -4161,24 +4173,24 @@
         <v>122</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>278</v>
+        <v>153</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>234</v>
+        <v>303</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>303</v>
+        <v>122</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>304</v>
@@ -4186,7 +4198,7 @@
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>305</v>
@@ -4194,45 +4206,45 @@
       <c r="C109" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D109" s="3" t="s">
-        <v>9</v>
+      <c r="D109" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>55</v>
+        <v>307</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>11</v>
+        <v>311</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>9</v>
@@ -4246,33 +4258,33 @@
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>244</v>
+        <v>11</v>
       </c>
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>9</v>
@@ -4281,18 +4293,18 @@
         <v>55</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>9</v>
@@ -4301,18 +4313,18 @@
         <v>55</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>9</v>
@@ -4321,61 +4333,61 @@
         <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>320</v>
+        <v>52</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>52</v>
+        <v>324</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="D117" s="5" t="s">
-        <v>234</v>
+        <v>326</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>122</v>
@@ -4386,133 +4398,133 @@
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>327</v>
+        <v>282</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>9</v>
+        <v>330</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>330</v>
+        <v>11</v>
       </c>
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>244</v>
+        <v>334</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>335</v>
+        <v>248</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>244</v>
+        <v>342</v>
       </c>
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>343</v>
+        <v>248</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>9</v>
@@ -4521,12 +4533,12 @@
         <v>122</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>348</v>
@@ -4538,7 +4550,7 @@
         <v>9</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>10</v>
+        <v>122</v>
       </c>
       <c r="F126" s="2" t="s">
         <v>350</v>
@@ -4546,76 +4558,76 @@
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="D128" s="4" t="s">
-        <v>151</v>
+        <v>356</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>234</v>
+        <v>359</v>
+      </c>
+      <c r="D129" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>11</v>
+        <v>360</v>
       </c>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>122</v>
@@ -4626,33 +4638,33 @@
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>9</v>
+        <v>364</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>10</v>
+        <v>122</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>364</v>
+        <v>11</v>
       </c>
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>9</v>
@@ -4661,58 +4673,58 @@
         <v>10</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>9</v>
@@ -4721,38 +4733,38 @@
         <v>10</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>52</v>
+        <v>377</v>
       </c>
     </row>
     <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>244</v>
+        <v>52</v>
       </c>
     </row>
     <row r="137" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>9</v>
@@ -4761,18 +4773,18 @@
         <v>55</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="138" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>9</v>
@@ -4781,107 +4793,107 @@
         <v>55</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="D139" s="4" t="s">
-        <v>151</v>
+        <v>385</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>384</v>
+        <v>52</v>
       </c>
     </row>
     <row r="140" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="D140" s="3" t="s">
-        <v>9</v>
+        <v>387</v>
+      </c>
+      <c r="D140" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>52</v>
+        <v>388</v>
       </c>
     </row>
     <row r="141" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="D141" s="4" t="s">
-        <v>151</v>
+        <v>390</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>389</v>
+        <v>52</v>
       </c>
     </row>
     <row r="142" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>234</v>
+        <v>392</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>109</v>
+        <v>365</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="D143" s="3" t="s">
-        <v>9</v>
+        <v>395</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4889,39 +4901,39 @@
         <v>109</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="145" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="146" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4929,10 +4941,10 @@
         <v>153</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>9</v>
@@ -4941,7 +4953,7 @@
         <v>55</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="147" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4949,10 +4961,10 @@
         <v>153</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>9</v>
@@ -4961,7 +4973,7 @@
         <v>55</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="148" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4969,19 +4981,19 @@
         <v>153</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="149" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4989,10 +5001,10 @@
         <v>153</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D149" s="3" t="s">
         <v>9</v>
@@ -5001,7 +5013,7 @@
         <v>122</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="150" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5009,10 +5021,10 @@
         <v>153</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>9</v>
@@ -5021,7 +5033,7 @@
         <v>122</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="151" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5029,10 +5041,10 @@
         <v>153</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D151" s="3" t="s">
         <v>9</v>
@@ -5041,7 +5053,7 @@
         <v>122</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="152" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5049,10 +5061,10 @@
         <v>153</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>9</v>
@@ -5061,7 +5073,7 @@
         <v>122</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="153" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5069,10 +5081,10 @@
         <v>153</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>9</v>
@@ -5081,7 +5093,7 @@
         <v>122</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="154" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5089,10 +5101,10 @@
         <v>153</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>9</v>
@@ -5101,18 +5113,18 @@
         <v>122</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="155" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>327</v>
+        <v>153</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D155" s="3" t="s">
         <v>9</v>
@@ -5121,18 +5133,18 @@
         <v>122</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="156" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>153</v>
+        <v>331</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>9</v>
@@ -5141,7 +5153,7 @@
         <v>122</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="157" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5149,10 +5161,10 @@
         <v>153</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>9</v>
@@ -5161,7 +5173,7 @@
         <v>122</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="158" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5169,10 +5181,10 @@
         <v>153</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>9</v>
@@ -5181,7 +5193,7 @@
         <v>122</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="159" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5189,10 +5201,10 @@
         <v>153</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>9</v>
@@ -5201,18 +5213,18 @@
         <v>122</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="160" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>9</v>
@@ -5221,18 +5233,18 @@
         <v>122</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="161" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>9</v>
@@ -5241,18 +5253,18 @@
         <v>122</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="162" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>9</v>
@@ -5261,18 +5273,18 @@
         <v>122</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="163" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>9</v>
@@ -5281,7 +5293,7 @@
         <v>122</v>
       </c>
       <c r="F163" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="164" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5289,19 +5301,19 @@
         <v>153</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E164" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="165" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5309,24 +5321,24 @@
         <v>153</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="166" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>462</v>
+        <v>153</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>463</v>
@@ -5338,7 +5350,7 @@
         <v>9</v>
       </c>
       <c r="E166" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F166" s="2" t="s">
         <v>465</v>
@@ -5346,33 +5358,33 @@
     </row>
     <row r="167" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>278</v>
+        <v>466</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="168" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>153</v>
+        <v>282</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>9</v>
@@ -5381,7 +5393,7 @@
         <v>122</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="169" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5389,10 +5401,10 @@
         <v>153</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>9</v>
@@ -5401,7 +5413,7 @@
         <v>122</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="170" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5409,10 +5421,10 @@
         <v>153</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D170" s="3" t="s">
         <v>9</v>
@@ -5421,7 +5433,7 @@
         <v>122</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="171" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5429,10 +5441,10 @@
         <v>153</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D171" s="3" t="s">
         <v>9</v>
@@ -5441,7 +5453,7 @@
         <v>122</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="172" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5449,10 +5461,10 @@
         <v>153</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D172" s="3" t="s">
         <v>9</v>
@@ -5461,7 +5473,7 @@
         <v>122</v>
       </c>
       <c r="F172" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="173" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5469,10 +5481,10 @@
         <v>153</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D173" s="3" t="s">
         <v>9</v>
@@ -5481,7 +5493,7 @@
         <v>122</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="174" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5489,10 +5501,10 @@
         <v>153</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D174" s="3" t="s">
         <v>9</v>
@@ -5501,7 +5513,7 @@
         <v>122</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="175" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5509,10 +5521,10 @@
         <v>153</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D175" s="3" t="s">
         <v>9</v>
@@ -5521,18 +5533,18 @@
         <v>122</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="176" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>278</v>
+        <v>153</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D176" s="3" t="s">
         <v>9</v>
@@ -5541,18 +5553,18 @@
         <v>122</v>
       </c>
       <c r="F176" s="2" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="177" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>201</v>
+        <v>282</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D177" s="3" t="s">
         <v>9</v>
@@ -5561,18 +5573,18 @@
         <v>122</v>
       </c>
       <c r="F177" s="2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="178" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>278</v>
+        <v>205</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D178" s="3" t="s">
         <v>9</v>
@@ -5581,38 +5593,38 @@
         <v>122</v>
       </c>
       <c r="F178" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="179" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>462</v>
+        <v>282</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D179" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F179" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="180" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D180" s="3" t="s">
         <v>9</v>
@@ -5621,11 +5633,31 @@
         <v>55</v>
       </c>
       <c r="F180" s="2" t="s">
-        <v>507</v>
+        <v>508</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="D181" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E181" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F181" s="2" t="s">
+        <v>511</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F180"/>
+  <autoFilter ref="A1:F181"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5633,7 +5665,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -5642,17 +5674,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5660,10 +5692,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5671,10 +5703,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5685,34 +5717,34 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B8">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="B9" s="13">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5726,10 +5758,10 @@
         <v>151</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5853,10 +5885,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B20">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -5865,55 +5897,55 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B22">
         <v>3</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E23">
         <v>7</v>
@@ -5921,86 +5953,103 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="B24">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>327</v>
+        <v>282</v>
       </c>
       <c r="B25">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E25">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="B27">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
         <v>2</v>
       </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
       <c r="E27">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>462</v>
+        <v>365</v>
       </c>
       <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>466</v>
+      </c>
+      <c r="B29">
         <v>3</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>0</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>0</v>
       </c>
-      <c r="E28">
+      <c r="E29">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Decide subscription tiers, economics, and billing stack (task #20)
Add docs/subscription-plan.md: the self-funding subscription design.

- Tiers: Free (Haiku, ~30 msgs/day, 1 companion) vs Other Plus
  $9.99/mo or $69.99/yr (Sonnet up to a daily cap then Haiku, all
  companions, natural voice).
- Unit-economics sheet: per-user monthly cost by usage band and model
  (Haiku/Sonnet/Llama 70B) and margin at $9.99 across web vs store fees;
  flags the heavy-Sonnet-user risk and the daily-cap mitigation.
- Billing stack: RevenueCat as the entitlement source of truth + Stripe
  Web Billing for the PWA (~97% take-home), Play/Apple unified via
  RevenueCat for the future wrapper.

Tracker updated. Implementation tasks #21 (backend entitlement + webhook
+ server-side model gating) and #22 (paywall + UI) follow once the price
and paid-model policy are confirmed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="526">
   <si>
     <t>Category</t>
   </si>
@@ -788,6 +788,15 @@
     <t>TBD</t>
   </si>
   <si>
+    <t>Subscription plan + economics</t>
+  </si>
+  <si>
+    <t>Decided tiers (Free vs Other Plus $9.99/mo / $69.99/yr), paid model policy (Sonnet-capped then Haiku), unit-economics + margin sheet, and billing stack (RevenueCat Web Billing + Stripe; Play/Apple via RevenueCat)</t>
+  </si>
+  <si>
+    <t>NEW; docs/subscription-plan.md (task #20); implementation pending #21/#22</t>
+  </si>
+  <si>
     <t>Payment integration</t>
   </si>
   <si>
@@ -1553,7 +1562,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 180 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 181 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -2025,7 +2034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F182"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3886,8 +3895,8 @@
       <c r="C93" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D93" s="5" t="s">
-        <v>238</v>
+      <c r="D93" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>10</v>
@@ -3898,27 +3907,27 @@
     </row>
     <row r="94" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="C94" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="D94" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>265</v>
@@ -3930,7 +3939,7 @@
         <v>9</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>267</v>
@@ -3938,7 +3947,7 @@
     </row>
     <row r="96" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>268</v>
@@ -3958,7 +3967,7 @@
     </row>
     <row r="97" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>271</v>
@@ -3973,32 +3982,32 @@
         <v>55</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>248</v>
+        <v>273</v>
       </c>
     </row>
     <row r="98" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>275</v>
+        <v>248</v>
       </c>
     </row>
     <row r="99" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>276</v>
@@ -4018,7 +4027,7 @@
     </row>
     <row r="100" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>279</v>
@@ -4038,33 +4047,33 @@
     </row>
     <row r="101" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B101" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="C101" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="D101" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F101" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="D101" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F101" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="102" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>9</v>
@@ -4078,27 +4087,27 @@
     </row>
     <row r="103" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>289</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>290</v>
@@ -4118,7 +4127,7 @@
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>293</v>
@@ -4138,7 +4147,7 @@
     </row>
     <row r="106" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>296</v>
@@ -4150,7 +4159,7 @@
         <v>9</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>298</v>
@@ -4158,7 +4167,7 @@
     </row>
     <row r="107" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>299</v>
@@ -4178,7 +4187,7 @@
     </row>
     <row r="108" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>153</v>
+        <v>285</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>302</v>
@@ -4198,7 +4207,7 @@
     </row>
     <row r="109" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>282</v>
+        <v>153</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>305</v>
@@ -4206,31 +4215,31 @@
       <c r="C109" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D109" s="5" t="s">
-        <v>238</v>
+      <c r="D109" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E109" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F109" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="F109" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="110" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B110" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C110" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="C110" s="2" t="s">
+      <c r="D110" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E110" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>311</v>
@@ -4238,7 +4247,7 @@
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>312</v>
@@ -4250,21 +4259,21 @@
         <v>9</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>11</v>
+        <v>314</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>9</v>
@@ -4278,33 +4287,33 @@
     </row>
     <row r="113" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>248</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>9</v>
@@ -4318,13 +4327,13 @@
     </row>
     <row r="115" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>9</v>
@@ -4333,18 +4342,18 @@
         <v>55</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="116" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>9</v>
@@ -4353,12 +4362,12 @@
         <v>55</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>324</v>
+        <v>52</v>
       </c>
     </row>
     <row r="117" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>325</v>
@@ -4370,41 +4379,41 @@
         <v>9</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>52</v>
+        <v>327</v>
       </c>
     </row>
     <row r="118" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>238</v>
+        <v>329</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="119" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>238</v>
@@ -4418,7 +4427,7 @@
     </row>
     <row r="120" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>331</v>
+        <v>285</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>332</v>
@@ -4426,19 +4435,19 @@
       <c r="C120" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D120" s="3" t="s">
-        <v>9</v>
+      <c r="D120" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>334</v>
+        <v>11</v>
       </c>
     </row>
     <row r="121" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>335</v>
@@ -4450,35 +4459,35 @@
         <v>9</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>248</v>
+        <v>337</v>
       </c>
     </row>
     <row r="122" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>339</v>
+        <v>248</v>
       </c>
     </row>
     <row r="123" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>340</v>
@@ -4490,7 +4499,7 @@
         <v>9</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F123" s="2" t="s">
         <v>342</v>
@@ -4498,7 +4507,7 @@
     </row>
     <row r="124" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>343</v>
@@ -4510,35 +4519,35 @@
         <v>9</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>248</v>
+        <v>345</v>
       </c>
     </row>
     <row r="125" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>347</v>
+        <v>248</v>
       </c>
     </row>
     <row r="126" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>348</v>
@@ -4558,27 +4567,27 @@
     </row>
     <row r="127" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="B127" s="2" t="s">
+      <c r="C127" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="C127" s="2" t="s">
+      <c r="D127" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F127" s="2" t="s">
         <v>353</v>
-      </c>
-      <c r="D127" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F127" s="2" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="128" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>355</v>
@@ -4590,7 +4599,7 @@
         <v>9</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F128" s="2" t="s">
         <v>357</v>
@@ -4598,7 +4607,7 @@
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>358</v>
@@ -4606,11 +4615,11 @@
       <c r="C129" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D129" s="4" t="s">
-        <v>151</v>
+      <c r="D129" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F129" s="2" t="s">
         <v>360</v>
@@ -4618,7 +4627,7 @@
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>361</v>
@@ -4626,25 +4635,25 @@
       <c r="C130" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="D130" s="5" t="s">
-        <v>238</v>
+      <c r="D130" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>11</v>
+        <v>363</v>
       </c>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>238</v>
@@ -4658,7 +4667,7 @@
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>366</v>
@@ -4666,19 +4675,19 @@
       <c r="C132" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="D132" s="3" t="s">
-        <v>9</v>
+      <c r="D132" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>10</v>
+        <v>122</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>368</v>
+        <v>11</v>
       </c>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>369</v>
@@ -4698,7 +4707,7 @@
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>372</v>
@@ -4710,7 +4719,7 @@
         <v>9</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F134" s="2" t="s">
         <v>374</v>
@@ -4718,7 +4727,7 @@
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>375</v>
@@ -4730,7 +4739,7 @@
         <v>9</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F135" s="2" t="s">
         <v>377</v>
@@ -4738,7 +4747,7 @@
     </row>
     <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>378</v>
@@ -4753,38 +4762,38 @@
         <v>10</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>52</v>
+        <v>380</v>
       </c>
     </row>
     <row r="137" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>248</v>
+        <v>52</v>
       </c>
     </row>
     <row r="138" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>9</v>
@@ -4798,13 +4807,13 @@
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>9</v>
@@ -4813,32 +4822,32 @@
         <v>55</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="140" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="D140" s="4" t="s">
-        <v>151</v>
+        <v>388</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>388</v>
+        <v>52</v>
       </c>
     </row>
     <row r="141" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>389</v>
@@ -4846,39 +4855,39 @@
       <c r="C141" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="D141" s="3" t="s">
-        <v>9</v>
+      <c r="D141" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>52</v>
+        <v>391</v>
       </c>
     </row>
     <row r="142" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="D142" s="4" t="s">
-        <v>151</v>
+        <v>393</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>393</v>
+        <v>52</v>
       </c>
     </row>
     <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>394</v>
@@ -4886,8 +4895,8 @@
       <c r="C143" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="D143" s="5" t="s">
-        <v>238</v>
+      <c r="D143" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>55</v>
@@ -4898,7 +4907,7 @@
     </row>
     <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>109</v>
+        <v>368</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>397</v>
@@ -4906,8 +4915,8 @@
       <c r="C144" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="D144" s="3" t="s">
-        <v>9</v>
+      <c r="D144" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>55</v>
@@ -4930,7 +4939,7 @@
         <v>9</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F145" s="2" t="s">
         <v>402</v>
@@ -4938,7 +4947,7 @@
     </row>
     <row r="146" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>403</v>
@@ -4950,7 +4959,7 @@
         <v>9</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F146" s="2" t="s">
         <v>405</v>
@@ -5010,7 +5019,7 @@
         <v>9</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F149" s="2" t="s">
         <v>414</v>
@@ -5138,7 +5147,7 @@
     </row>
     <row r="156" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>331</v>
+        <v>153</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>433</v>
@@ -5158,7 +5167,7 @@
     </row>
     <row r="157" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>153</v>
+        <v>334</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>436</v>
@@ -5238,7 +5247,7 @@
     </row>
     <row r="161" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>448</v>
@@ -5258,7 +5267,7 @@
     </row>
     <row r="162" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>451</v>
@@ -5278,7 +5287,7 @@
     </row>
     <row r="163" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>454</v>
@@ -5298,7 +5307,7 @@
     </row>
     <row r="164" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>457</v>
@@ -5330,7 +5339,7 @@
         <v>9</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F165" s="2" t="s">
         <v>462</v>
@@ -5350,7 +5359,7 @@
         <v>9</v>
       </c>
       <c r="E166" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F166" s="2" t="s">
         <v>465</v>
@@ -5358,27 +5367,27 @@
     </row>
     <row r="167" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B167" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="B167" s="2" t="s">
+      <c r="C167" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="C167" s="2" t="s">
+      <c r="D167" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F167" s="2" t="s">
         <v>468</v>
-      </c>
-      <c r="D167" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E167" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F167" s="2" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="168" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>282</v>
+        <v>469</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>470</v>
@@ -5390,7 +5399,7 @@
         <v>9</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F168" s="2" t="s">
         <v>472</v>
@@ -5398,7 +5407,7 @@
     </row>
     <row r="169" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>153</v>
+        <v>285</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>473</v>
@@ -5558,7 +5567,7 @@
     </row>
     <row r="177" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>282</v>
+        <v>153</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>497</v>
@@ -5578,7 +5587,7 @@
     </row>
     <row r="178" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>205</v>
+        <v>285</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>500</v>
@@ -5598,7 +5607,7 @@
     </row>
     <row r="179" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>282</v>
+        <v>205</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>503</v>
@@ -5618,7 +5627,7 @@
     </row>
     <row r="180" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>466</v>
+        <v>285</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>506</v>
@@ -5630,7 +5639,7 @@
         <v>9</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F180" s="2" t="s">
         <v>508</v>
@@ -5638,7 +5647,7 @@
     </row>
     <row r="181" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>509</v>
@@ -5656,8 +5665,28 @@
         <v>511</v>
       </c>
     </row>
+    <row r="182" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="D182" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E182" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F182" s="2" t="s">
+        <v>514</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F181"/>
+  <autoFilter ref="A1:F182"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5674,17 +5703,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5692,10 +5721,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5703,10 +5732,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C6" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5717,7 +5746,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5728,23 +5757,23 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B9" s="13">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5761,7 +5790,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5939,7 +5968,7 @@
         <v>239</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -5948,12 +5977,12 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B24">
         <v>7</v>
@@ -5970,7 +5999,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B25">
         <v>18</v>
@@ -5987,7 +6016,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B26">
         <v>8</v>
@@ -6004,7 +6033,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B27">
         <v>2</v>
@@ -6021,7 +6050,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -6038,7 +6067,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B29">
         <v>3</v>

</xml_diff>

<commit_message>
Regenerate feature xlsx (184 features, 168 Built)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="535">
   <si>
     <t>Category</t>
   </si>
@@ -1166,6 +1166,15 @@
     <t>NEW; config AI_MODEL, prompt.buildSystemBlocks, ai.js systemBlocks, worker forwards blocks</t>
   </si>
   <si>
+    <t>On-device AI (token-free)</t>
+  </si>
+  <si>
+    <t>Opt-in: companions run on a small model in the browser via WebGPU/WebLLM (Llama 3.2 3B) — real replies at ZERO token cost, private, offline. web-llm is dynamically imported (separate lazy chunk, no main-bundle bloat); precedence on-device &gt; proxy &gt; placeholder; WebGPU capability-detected with graceful fallback; Settings toggle + download progress; 'On-device' live indicator</t>
+  </si>
+  <si>
+    <t>NEW (task #19); lib/ondevice.js, ai.js askCompanion/proactive routing, Settings section. Real inference needs a WebGPU device (untested in CI)</t>
+  </si>
+  <si>
     <t>Accounts &amp; auth</t>
   </si>
   <si>
@@ -1580,7 +1589,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 183 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 184 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -2052,7 +2061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4817,10 +4826,10 @@
         <v>9</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>52</v>
+        <v>386</v>
       </c>
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4828,19 +4837,19 @@
         <v>371</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>248</v>
+        <v>52</v>
       </c>
     </row>
     <row r="140" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4848,10 +4857,10 @@
         <v>371</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>9</v>
@@ -4868,10 +4877,10 @@
         <v>371</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>9</v>
@@ -4880,7 +4889,7 @@
         <v>55</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="142" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4888,19 +4897,19 @@
         <v>371</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="D142" s="4" t="s">
-        <v>151</v>
+        <v>394</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>394</v>
+        <v>52</v>
       </c>
     </row>
     <row r="143" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4913,14 +4922,14 @@
       <c r="C143" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="D143" s="3" t="s">
-        <v>9</v>
+      <c r="D143" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>52</v>
+        <v>397</v>
       </c>
     </row>
     <row r="144" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4928,19 +4937,19 @@
         <v>371</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D144" s="4" t="s">
-        <v>151</v>
+        <v>399</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>399</v>
+        <v>52</v>
       </c>
     </row>
     <row r="145" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4953,8 +4962,8 @@
       <c r="C145" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="D145" s="5" t="s">
-        <v>238</v>
+      <c r="D145" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>55</v>
@@ -4973,11 +4982,11 @@
       <c r="C146" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="D146" s="3" t="s">
-        <v>9</v>
+      <c r="D146" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="F146" s="2" t="s">
         <v>405</v>
@@ -4985,7 +4994,7 @@
     </row>
     <row r="147" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>109</v>
+        <v>371</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>406</v>
@@ -4997,7 +5006,7 @@
         <v>9</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F147" s="2" t="s">
         <v>408</v>
@@ -5017,7 +5026,7 @@
         <v>9</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F148" s="2" t="s">
         <v>411</v>
@@ -5025,7 +5034,7 @@
     </row>
     <row r="149" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>412</v>
@@ -5037,7 +5046,7 @@
         <v>9</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F149" s="2" t="s">
         <v>414</v>
@@ -5097,7 +5106,7 @@
         <v>9</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F152" s="2" t="s">
         <v>423</v>
@@ -5225,7 +5234,7 @@
     </row>
     <row r="159" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>337</v>
+        <v>153</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>442</v>
@@ -5245,7 +5254,7 @@
     </row>
     <row r="160" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>153</v>
+        <v>337</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>445</v>
@@ -5325,7 +5334,7 @@
     </row>
     <row r="164" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>457</v>
@@ -5345,7 +5354,7 @@
     </row>
     <row r="165" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>460</v>
@@ -5365,7 +5374,7 @@
     </row>
     <row r="166" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>463</v>
@@ -5385,7 +5394,7 @@
     </row>
     <row r="167" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>466</v>
@@ -5417,7 +5426,7 @@
         <v>9</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F168" s="2" t="s">
         <v>471</v>
@@ -5437,7 +5446,7 @@
         <v>9</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F169" s="2" t="s">
         <v>474</v>
@@ -5445,27 +5454,27 @@
     </row>
     <row r="170" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B170" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="B170" s="2" t="s">
+      <c r="C170" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="C170" s="2" t="s">
+      <c r="D170" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F170" s="2" t="s">
         <v>477</v>
-      </c>
-      <c r="D170" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E170" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F170" s="2" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="171" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>288</v>
+        <v>478</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>479</v>
@@ -5477,7 +5486,7 @@
         <v>9</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F171" s="2" t="s">
         <v>481</v>
@@ -5485,7 +5494,7 @@
     </row>
     <row r="172" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>153</v>
+        <v>288</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>482</v>
@@ -5645,7 +5654,7 @@
     </row>
     <row r="180" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>288</v>
+        <v>153</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>506</v>
@@ -5665,7 +5674,7 @@
     </row>
     <row r="181" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>205</v>
+        <v>288</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>509</v>
@@ -5685,7 +5694,7 @@
     </row>
     <row r="182" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>288</v>
+        <v>205</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>512</v>
@@ -5705,7 +5714,7 @@
     </row>
     <row r="183" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>475</v>
+        <v>288</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>515</v>
@@ -5717,7 +5726,7 @@
         <v>9</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F183" s="2" t="s">
         <v>517</v>
@@ -5725,7 +5734,7 @@
     </row>
     <row r="184" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="B184" s="2" t="s">
         <v>518</v>
@@ -5743,8 +5752,28 @@
         <v>520</v>
       </c>
     </row>
+    <row r="185" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="D185" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E185" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F185" s="2" t="s">
+        <v>523</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F184"/>
+  <autoFilter ref="A1:F185"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5761,17 +5790,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5779,10 +5808,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5790,10 +5819,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C6" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5804,7 +5833,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5815,23 +5844,23 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B9" s="13">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5848,7 +5877,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -6111,7 +6140,7 @@
         <v>371</v>
       </c>
       <c r="B28">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -6120,12 +6149,12 @@
         <v>1</v>
       </c>
       <c r="E28">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="B29">
         <v>3</v>

</xml_diff>

<commit_message>
Add broad roadmap features to the tracker/spreadsheet
Log the owner-approved "for everyone" roadmap as Future entries (Play &
activities parked at P3): voice call mode, year-with-you recap, real-life
milestone celebration, companion cards (shareable image), companion-made
gifts, guided journaling, gentle goals/accountability, daily check-in
streak, seasonal/holiday moments, companion voice notes, and photo
moments. Regenerate OTHER_App_Features.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="579">
   <si>
     <t>Category</t>
   </si>
@@ -1607,10 +1607,121 @@
     <t>NEW; claimBeat() gates milestone/vulnerability/rift/occasion/curiosity</t>
   </si>
   <si>
+    <t>Roadmap</t>
+  </si>
+  <si>
+    <t>Voice call mode</t>
+  </si>
+  <si>
+    <t>Hands-free continuous 'phone call' with a companion — call screen, back-and-forth speech (reuses TTS + speech recognition)</t>
+  </si>
+  <si>
+    <t>PLANNED; builds on lib/voice.js</t>
+  </si>
+  <si>
+    <t>Year-with-you recap</t>
+  </si>
+  <si>
+    <t>Periodic companion-narrated relationship recap: milestones, inside jokes, moods, how the bond grew; shareable</t>
+  </si>
+  <si>
+    <t>PLANNED; uses lore/jokes/bond/mood already tracked</t>
+  </si>
+  <si>
+    <t>Real-life milestone celebration</t>
+  </si>
+  <si>
+    <t>Companion remembers + shows up for the user's real big days (birthday, anniversaries, mentioned events)</t>
+  </si>
+  <si>
+    <t>PLANNED; builds on occasion.js + memory</t>
+  </si>
+  <si>
+    <t>Companion cards (shareable image)</t>
+  </si>
+  <si>
+    <t>Generate a shareable image: companion avatar + a memorable line, with ToS 7.3 attribution baked in (growth loop)</t>
+  </si>
+  <si>
+    <t>PLANNED; canvas render of Avatar/SquishyBlob + quote</t>
+  </si>
+  <si>
+    <t>Companion-made gifts</t>
+  </si>
+  <si>
+    <t>Companion writes a poem, makes a playlist, or 'draws' (markdown art) on special moments</t>
+  </si>
+  <si>
+    <t>PLANNED; AI generation + keepsake in Story so far</t>
+  </si>
+  <si>
+    <t>Guided journaling</t>
+  </si>
+  <si>
+    <t>Companion-prompted reflective journaling with a private, searchable user journal</t>
+  </si>
+  <si>
+    <t>PLANNED; distinct from companion journals; reuse search</t>
+  </si>
+  <si>
+    <t>Gentle goals &amp; accountability</t>
+  </si>
+  <si>
+    <t>Set a goal; companion checks in and celebrates progress</t>
+  </si>
+  <si>
+    <t>PLANNED; reuses reminders + check-ins</t>
+  </si>
+  <si>
+    <t>Daily check-in streak</t>
+  </si>
+  <si>
+    <t>Warm once-a-day 'how are you?' building a streak + visible mood history</t>
+  </si>
+  <si>
+    <t>PLANNED; reuses mood tracking</t>
+  </si>
+  <si>
+    <t>Seasonal &amp; holiday moments</t>
+  </si>
+  <si>
+    <t>The Space + companions react to seasons / holidays / weather year-round</t>
+  </si>
+  <si>
+    <t>PLANNED; builds on occasion.js + weatherNow()</t>
+  </si>
+  <si>
+    <t>Companion voice notes</t>
+  </si>
+  <si>
+    <t>Occasional spoken messages instead of text (natural voice when configured)</t>
+  </si>
+  <si>
+    <t>PLANNED; lib/voice.js</t>
+  </si>
+  <si>
+    <t>Photo moments</t>
+  </si>
+  <si>
+    <t>User shares a photo; companion reacts warmly (vision model — premium due to cost)</t>
+  </si>
+  <si>
+    <t>PLANNED; needs vision-capable model, gate to premium</t>
+  </si>
+  <si>
+    <t>Play &amp; activities together</t>
+  </si>
+  <si>
+    <t>Mini-games (would-you-rather, 20 questions, story-building) + watch/read-along recommendations</t>
+  </si>
+  <si>
+    <t>PARKED by owner — revisit later</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 186 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 198 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -1622,13 +1733,13 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>91%</t>
+    <t>86%</t>
   </si>
   <si>
     <t>4%</t>
   </si>
   <si>
-    <t>5%</t>
+    <t>11%</t>
   </si>
   <si>
     <t>Total</t>
@@ -2082,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F187"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5833,8 +5944,248 @@
         <v>530</v>
       </c>
     </row>
+    <row r="188" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B188" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="C188" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="D188" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F188" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E189" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F189" s="2" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E190" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F190" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F191" s="2" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E192" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F192" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="D193" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E193" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F193" s="2" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F194" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E195" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F195" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E196" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F196" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E197" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F197" s="2" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E198" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F198" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E199" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F199" s="2" t="s">
+        <v>567</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F187"/>
+  <autoFilter ref="A1:F199"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5842,7 +6193,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -5851,17 +6202,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>531</v>
+        <v>568</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>532</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>533</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5869,10 +6220,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>534</v>
+        <v>571</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>535</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5883,7 +6234,7 @@
         <v>170</v>
       </c>
       <c r="C6" t="s">
-        <v>536</v>
+        <v>573</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5894,7 +6245,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>537</v>
+        <v>574</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5902,26 +6253,26 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>538</v>
+        <v>575</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>539</v>
+        <v>576</v>
       </c>
       <c r="B9" s="13">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>540</v>
+        <v>577</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>541</v>
+        <v>578</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5938,7 +6289,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>539</v>
+        <v>576</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -6245,6 +6596,23 @@
       </c>
       <c r="E30">
         <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>531</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>12</v>
+      </c>
+      <c r="E31">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Year-with-you recap keepsake (#24)
A companion-narrated look back at the relationship, built from data the
app already keeps: how long you've known each other, closeness per
companion, shared moments (lore), inside jokes, and letters — with a
copy/share button (attribution baked in). A gentle once-a-month companion
nudge points to it, gated by claimBeat so it never floods.

- screens/Recap.jsx (uses innerlife closenessStage/knownDuration)
- Chat: 'recap' panel + "✨ Your recap" menu item + monthly nudge effect

Verified in a real browser: recap renders intro, closeness, moments,
inside jokes, and letters; Share copies. No runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1616,18 +1616,18 @@
     <t>NEW (task #23); components/CallScreen.jsx, voice.speakAsAsync/stopSpeaking, Chat call state machine; group call per owner request</t>
   </si>
   <si>
+    <t>Year-with-you recap</t>
+  </si>
+  <si>
+    <t>Companion-narrated keepsake: how long you've known each other, closeness per companion, shared moments (lore), inside jokes, letters; copy/share with attribution; gentle once-a-month nudge</t>
+  </si>
+  <si>
+    <t>NEW (task #24); screens/Recap.jsx, menu + panel + monthly nudge</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Year-with-you recap</t>
-  </si>
-  <si>
-    <t>Periodic companion-narrated relationship recap: milestones, inside jokes, moods, how the bond grew; shareable</t>
-  </si>
-  <si>
-    <t>PLANNED; uses lore/jokes/bond/mood already tracked</t>
-  </si>
-  <si>
     <t>Real-life milestone celebration</t>
   </si>
   <si>
@@ -1733,7 +1733,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>86%</t>
+    <t>87%</t>
   </si>
   <si>
     <t>4%</t>
@@ -5966,27 +5966,27 @@
     </row>
     <row r="189" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B189" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="B189" s="2" t="s">
+      <c r="C189" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="C189" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="D189" s="5" t="s">
-        <v>238</v>
+      <c r="D189" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F189" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="190" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>538</v>
@@ -6006,7 +6006,7 @@
     </row>
     <row r="191" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>541</v>
@@ -6026,7 +6026,7 @@
     </row>
     <row r="192" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>544</v>
@@ -6046,7 +6046,7 @@
     </row>
     <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>547</v>
@@ -6066,7 +6066,7 @@
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>550</v>
@@ -6086,7 +6086,7 @@
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>553</v>
@@ -6106,7 +6106,7 @@
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>556</v>
@@ -6126,7 +6126,7 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>559</v>
@@ -6146,7 +6146,7 @@
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>562</v>
@@ -6166,7 +6166,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>565</v>
@@ -6231,7 +6231,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C6" t="s">
         <v>573</v>
@@ -6253,7 +6253,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
         <v>575</v>
@@ -6382,7 +6382,7 @@
         <v>153</v>
       </c>
       <c r="B18">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -6391,7 +6391,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -6600,7 +6600,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -6609,10 +6609,10 @@
         <v>0</v>
       </c>
       <c r="D31">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E31">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add real-life milestone celebrations (#25)
A companion shows up in chat for the user's real big days: their birthday
(from DOB), "we met" anniversaries (1/3/6 months, then yearly), and dated
events they mentioned (memories carrying an `at` timestamp). Each fires at
most once, tracked in localStorage; milestones bypass the shared beat
coordinator since they're rare and special.

- occasion.js: pendingMilestones() + monthsLabel()
- Chat: milestone celebration effect

Verified in a real browser: a same-day birthday triggers a warm message,
and the dedup key prevents re-firing. No runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1625,18 +1625,18 @@
     <t>NEW (task #24); screens/Recap.jsx, menu + panel + monthly nudge</t>
   </si>
   <si>
+    <t>Real-life milestone celebration</t>
+  </si>
+  <si>
+    <t>A companion shows up in chat for the user's real big days: birthday (from DOB), 'we met' anniversaries (1/3/6 months then yearly), and dated events the user mentioned (memories with an 'at' date). Each fires once (deduped)</t>
+  </si>
+  <si>
+    <t>NEW (task #25); occasion.pendingMilestones/monthsLabel, Chat celebration effect</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Real-life milestone celebration</t>
-  </si>
-  <si>
-    <t>Companion remembers + shows up for the user's real big days (birthday, anniversaries, mentioned events)</t>
-  </si>
-  <si>
-    <t>PLANNED; builds on occasion.js + memory</t>
-  </si>
-  <si>
     <t>Companion cards (shareable image)</t>
   </si>
   <si>
@@ -1739,7 +1739,7 @@
     <t>4%</t>
   </si>
   <si>
-    <t>10%</t>
+    <t>9%</t>
   </si>
   <si>
     <t>Total</t>
@@ -5986,27 +5986,27 @@
     </row>
     <row r="190" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B190" s="2" t="s">
         <v>537</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="C190" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="C190" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="D190" s="5" t="s">
-        <v>238</v>
+      <c r="D190" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E190" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F190" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="191" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>541</v>
@@ -6026,7 +6026,7 @@
     </row>
     <row r="192" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>544</v>
@@ -6046,7 +6046,7 @@
     </row>
     <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>547</v>
@@ -6066,7 +6066,7 @@
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>550</v>
@@ -6086,7 +6086,7 @@
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>553</v>
@@ -6106,7 +6106,7 @@
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>556</v>
@@ -6126,7 +6126,7 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>559</v>
@@ -6146,7 +6146,7 @@
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>562</v>
@@ -6166,7 +6166,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>565</v>
@@ -6231,7 +6231,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
         <v>573</v>
@@ -6253,7 +6253,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
         <v>575</v>
@@ -6382,7 +6382,7 @@
         <v>153</v>
       </c>
       <c r="B18">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -6391,7 +6391,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -6600,7 +6600,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -6609,10 +6609,10 @@
         <v>0</v>
       </c>
       <c r="D31">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E31">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add shareable companion cards (#26)
Tap 🖼 on any companion message to generate a 1080px shareable card — a
cosmic orb with the companion's constellation sigil, the quoted line, and
ToS §7.3 attribution baked in — then share via the native share sheet or
download. Pure canvas (no network, no image-AI), so it's a zero-cost
growth loop.

- lib/card.js: makeCardBlob() (canvas PNG) + shareOrDownloadCard()
- Chat: 🖼 control on assistant messages

Verified in a real browser: the button generates and downloads a valid
~760KB PNG; the card renders the orb, name, quote, and attribution. No
runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="580">
   <si>
     <t>Category</t>
   </si>
@@ -1634,18 +1634,21 @@
     <t>NEW (task #25); occasion.pendingMilestones/monthsLabel, Chat celebration effect</t>
   </si>
   <si>
+    <t>Shareable</t>
+  </si>
+  <si>
+    <t>Companion cards (shareable image)</t>
+  </si>
+  <si>
+    <t>Tap 🖼 on any companion message to make a 1080px card — cosmic orb + their constellation + the quote + ToS 7.3 attribution — and share (native share sheet) or download. Pure canvas, no cost (growth loop)</t>
+  </si>
+  <si>
+    <t>NEW (task #26); lib/card.js makeCardBlob/shareOrDownloadCard, message control</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Companion cards (shareable image)</t>
-  </si>
-  <si>
-    <t>Generate a shareable image: companion avatar + a memorable line, with ToS 7.3 attribution baked in (growth loop)</t>
-  </si>
-  <si>
-    <t>PLANNED; canvas render of Avatar/SquishyBlob + quote</t>
-  </si>
-  <si>
     <t>Companion-made gifts</t>
   </si>
   <si>
@@ -1733,7 +1736,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>87%</t>
+    <t>88%</t>
   </si>
   <si>
     <t>4%</t>
@@ -6014,8 +6017,8 @@
       <c r="C191" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="D191" s="5" t="s">
-        <v>238</v>
+      <c r="D191" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E191" s="2" t="s">
         <v>55</v>
@@ -6026,13 +6029,13 @@
     </row>
     <row r="192" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>238</v>
@@ -6041,18 +6044,18 @@
         <v>122</v>
       </c>
       <c r="F192" s="2" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>238</v>
@@ -6061,18 +6064,18 @@
         <v>55</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>238</v>
@@ -6081,18 +6084,18 @@
         <v>122</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>238</v>
@@ -6101,18 +6104,18 @@
         <v>122</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>238</v>
@@ -6121,18 +6124,18 @@
         <v>122</v>
       </c>
       <c r="F196" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>238</v>
@@ -6141,18 +6144,18 @@
         <v>122</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>238</v>
@@ -6161,18 +6164,18 @@
         <v>122</v>
       </c>
       <c r="F198" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>238</v>
@@ -6181,7 +6184,7 @@
         <v>313</v>
       </c>
       <c r="F199" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
   </sheetData>
@@ -6193,7 +6196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -6202,17 +6205,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -6220,10 +6223,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -6231,10 +6234,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C6" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -6245,7 +6248,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -6253,26 +6256,26 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B9" s="13">
         <v>198</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -6289,7 +6292,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -6603,16 +6606,33 @@
         <v>540</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>9</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>544</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>8</v>
+      </c>
+      <c r="E32">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add guided journaling — private user journal (#27)
A private journal distinct from companions' journals: a rotating daily
reflective prompt, free-write entries, a browsable + searchable history,
and delete. Entries persist in the session (local + synced) and are NEVER
sent to the AI — it's the user's private space.

- lib/journal.js (prompts + entry helpers), screens/Journal.jsx
- Chat: journal state threaded into persistence + 'journal' panel +
  "📓 Journal" menu item; App restore/applyState carry it too

Verified in a real browser: writing saves, the entry persists across a
real reload, search filters, and there are no runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="581">
   <si>
     <t>Category</t>
   </si>
@@ -1658,13 +1658,16 @@
     <t>PLANNED; AI generation + keepsake in Story so far</t>
   </si>
   <si>
+    <t>Daily life</t>
+  </si>
+  <si>
     <t>Guided journaling</t>
   </si>
   <si>
-    <t>Companion-prompted reflective journaling with a private, searchable user journal</t>
-  </si>
-  <si>
-    <t>PLANNED; distinct from companion journals; reuse search</t>
+    <t>Private user journal (distinct from companion journals): a rotating daily reflective prompt, free-write entries, browsable + searchable, delete. Persists + syncs in the session; NEVER sent to the AI</t>
+  </si>
+  <si>
+    <t>NEW (task #27); lib/journal.js, screens/Journal.jsx, menu + panel, threaded App&lt;-&gt;Chat persist</t>
   </si>
   <si>
     <t>Gentle goals &amp; accountability</t>
@@ -1742,7 +1745,7 @@
     <t>4%</t>
   </si>
   <si>
-    <t>9%</t>
+    <t>8%</t>
   </si>
   <si>
     <t>Total</t>
@@ -6049,22 +6052,22 @@
     </row>
     <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>549</v>
-      </c>
-      <c r="D193" s="5" t="s">
-        <v>238</v>
+        <v>550</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E193" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6072,10 +6075,10 @@
         <v>544</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>238</v>
@@ -6084,7 +6087,7 @@
         <v>122</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6092,10 +6095,10 @@
         <v>544</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>238</v>
@@ -6104,7 +6107,7 @@
         <v>122</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6112,10 +6115,10 @@
         <v>544</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>238</v>
@@ -6124,7 +6127,7 @@
         <v>122</v>
       </c>
       <c r="F196" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6132,10 +6135,10 @@
         <v>544</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>238</v>
@@ -6144,7 +6147,7 @@
         <v>122</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6152,10 +6155,10 @@
         <v>544</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>238</v>
@@ -6164,7 +6167,7 @@
         <v>122</v>
       </c>
       <c r="F198" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6172,10 +6175,10 @@
         <v>544</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>238</v>
@@ -6184,7 +6187,7 @@
         <v>313</v>
       </c>
       <c r="F199" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>
@@ -6196,7 +6199,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -6205,17 +6208,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -6223,10 +6226,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -6234,10 +6237,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -6248,7 +6251,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -6256,26 +6259,26 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B9" s="13">
         <v>198</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -6292,7 +6295,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -6629,10 +6632,27 @@
         <v>0</v>
       </c>
       <c r="D32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E32">
-        <v>8</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>548</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add companion-made gifts — poem / playlist / art (#28)
On rare close moments a companion makes the user a small creative gift —
a short poem, a tiny playlist, or text/ASCII art — generated in-character
(AI, with an offline template fallback) and saved as a keepsake in "Your
story so far".

- ai.generateGift + offlineGift
- innerlife: giftDue / giftKindFor / addGift (kind picked from personality)
- Chat: budgeted inner-life beat (after letters) posts a short note + saves
- StorySoFar: 🎁 Gifts section (monospace for art)

Verified in a real browser: a seeded gift renders in Story so far. No
runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1646,30 +1646,30 @@
     <t>NEW (task #26); lib/card.js makeCardBlob/shareOrDownloadCard, message control</t>
   </si>
   <si>
+    <t>Companion-made gifts</t>
+  </si>
+  <si>
+    <t>On rare close moments a companion makes a poem, a tiny playlist, or text/ASCII art (in-character, AI with offline fallback), saved as a keepsake in 'Your story so far'</t>
+  </si>
+  <si>
+    <t>NEW (task #28); ai.generateGift, innerlife.giftDue/giftKindFor/addGift, budgeted inner-life beat, StorySoFar Gifts section</t>
+  </si>
+  <si>
+    <t>Daily life</t>
+  </si>
+  <si>
+    <t>Guided journaling</t>
+  </si>
+  <si>
+    <t>Private user journal (distinct from companion journals): a rotating daily reflective prompt, free-write entries, browsable + searchable, delete. Persists + syncs in the session; NEVER sent to the AI</t>
+  </si>
+  <si>
+    <t>NEW (task #27); lib/journal.js, screens/Journal.jsx, menu + panel, threaded App&lt;-&gt;Chat persist</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Companion-made gifts</t>
-  </si>
-  <si>
-    <t>Companion writes a poem, makes a playlist, or 'draws' (markdown art) on special moments</t>
-  </si>
-  <si>
-    <t>PLANNED; AI generation + keepsake in Story so far</t>
-  </si>
-  <si>
-    <t>Daily life</t>
-  </si>
-  <si>
-    <t>Guided journaling</t>
-  </si>
-  <si>
-    <t>Private user journal (distinct from companion journals): a rotating daily reflective prompt, free-write entries, browsable + searchable, delete. Persists + syncs in the session; NEVER sent to the AI</t>
-  </si>
-  <si>
-    <t>NEW (task #27); lib/journal.js, screens/Journal.jsx, menu + panel, threaded App&lt;-&gt;Chat persist</t>
-  </si>
-  <si>
     <t>Gentle goals &amp; accountability</t>
   </si>
   <si>
@@ -1739,7 +1739,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>88%</t>
+    <t>89%</t>
   </si>
   <si>
     <t>4%</t>
@@ -6032,33 +6032,33 @@
     </row>
     <row r="192" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B192" s="2" t="s">
         <v>544</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="C192" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="C192" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="D192" s="5" t="s">
-        <v>238</v>
+      <c r="D192" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E192" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F192" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="193" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B193" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="B193" s="2" t="s">
+      <c r="C193" s="2" t="s">
         <v>549</v>
-      </c>
-      <c r="C193" s="2" t="s">
-        <v>550</v>
       </c>
       <c r="D193" s="3" t="s">
         <v>9</v>
@@ -6067,12 +6067,12 @@
         <v>55</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>552</v>
@@ -6092,7 +6092,7 @@
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>555</v>
@@ -6112,7 +6112,7 @@
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>558</v>
@@ -6132,7 +6132,7 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>561</v>
@@ -6152,7 +6152,7 @@
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>564</v>
@@ -6172,7 +6172,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>567</v>
@@ -6237,7 +6237,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
         <v>575</v>
@@ -6259,7 +6259,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
         <v>577</v>
@@ -6388,7 +6388,7 @@
         <v>153</v>
       </c>
       <c r="B18">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -6397,7 +6397,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -6623,36 +6623,36 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E32">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="B33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add gentle goals & accountability (#29)
Set goals you're working toward; a companion checks in kindly every few
days (gated, never naggy) and celebrates when you complete one.

- lib/goals.js (CRUD + goalToNudge/markNudged), screens/Goals.jsx
- Chat: goals threaded into persistence; check-in nudge effect +
  completion-celebration effect; "🌱 Goals" menu item + panel
- App restore/applyState carry goals

Verified in a real browser: add a goal, complete it -> companion
celebrates in chat, and it persists across reload. No runtime errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1667,18 +1667,18 @@
     <t>NEW (task #27); lib/journal.js, screens/Journal.jsx, menu + panel, threaded App&lt;-&gt;Chat persist</t>
   </si>
   <si>
+    <t>Gentle goals &amp; accountability</t>
+  </si>
+  <si>
+    <t>Set goals you're working toward; a companion checks in kindly (every few days, gated) and celebrates when you complete one. Add/complete/remove; persists + syncs</t>
+  </si>
+  <si>
+    <t>NEW (task #29); lib/goals.js, screens/Goals.jsx, Chat nudge + completion effects, menu + panel</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Gentle goals &amp; accountability</t>
-  </si>
-  <si>
-    <t>Set a goal; companion checks in and celebrates progress</t>
-  </si>
-  <si>
-    <t>PLANNED; reuses reminders + check-ins</t>
-  </si>
-  <si>
     <t>Daily check-in streak</t>
   </si>
   <si>
@@ -1745,7 +1745,7 @@
     <t>4%</t>
   </si>
   <si>
-    <t>8%</t>
+    <t>7%</t>
   </si>
   <si>
     <t>Total</t>
@@ -6072,27 +6072,27 @@
     </row>
     <row r="194" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B194" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="B194" s="2" t="s">
+      <c r="C194" s="2" t="s">
         <v>552</v>
       </c>
-      <c r="C194" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="D194" s="5" t="s">
-        <v>238</v>
+      <c r="D194" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E194" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>555</v>
@@ -6112,7 +6112,7 @@
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>558</v>
@@ -6132,7 +6132,7 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>561</v>
@@ -6152,7 +6152,7 @@
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>564</v>
@@ -6172,7 +6172,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>567</v>
@@ -6237,7 +6237,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C6" t="s">
         <v>575</v>
@@ -6259,7 +6259,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
         <v>577</v>
@@ -6626,7 +6626,7 @@
         <v>547</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -6635,12 +6635,12 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -6649,10 +6649,10 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add daily check-in streak (#30)
A warm once-a-day "how are you?" card appears in chat. Tapping a mood
(great/good/okay/low/anxious) records a no-pressure streak and a 60-day
mood history, logs the mood to the backend when signed in, and resolves
the card to a streak acknowledgement. A keepsake panel (CheckIn screen,
reachable from the chat menu) shows the current streak, recent moods as a
swatch grid, and an overall mood breakdown.

- src/lib/checkin.js: dayStr, CHECKIN_MOODS, moodColor, checkinDue, recordCheckin
- src/screens/CheckIn.jsx: keepsake panel
- src/screens/Chat.jsx: check-in effect, answerCheckin, card render, panel, menu item
- src/App.jsx: thread checkins through restore + applyState persistence
- docs: tracker row -> Built, regenerated xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1676,18 +1676,18 @@
     <t>NEW (task #29); lib/goals.js, screens/Goals.jsx, Chat nudge + completion effects, menu + panel</t>
   </si>
   <si>
+    <t>Daily check-in streak</t>
+  </si>
+  <si>
+    <t>Warm once-a-day 'how are you?' card in chat; tap a mood (great/good/okay/low/anxious) to record a no-pressure streak + 60-day mood history; keepsake panel with streak, recent moods, and an overall breakdown; logs mood to backend when signed in</t>
+  </si>
+  <si>
+    <t>NEW (task #30); lib/checkin.js, screens/CheckIn.jsx, Chat checkin card + answerCheckin + panel + menu, threaded App&lt;-&gt;Chat persist</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Daily check-in streak</t>
-  </si>
-  <si>
-    <t>Warm once-a-day 'how are you?' building a streak + visible mood history</t>
-  </si>
-  <si>
-    <t>PLANNED; reuses mood tracking</t>
-  </si>
-  <si>
     <t>Seasonal &amp; holiday moments</t>
   </si>
   <si>
@@ -1739,7 +1739,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>89%</t>
+    <t>90%</t>
   </si>
   <si>
     <t>4%</t>
@@ -6092,27 +6092,27 @@
     </row>
     <row r="195" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B195" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="B195" s="2" t="s">
+      <c r="C195" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="C195" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="D195" s="5" t="s">
-        <v>238</v>
+      <c r="D195" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="196" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>558</v>
@@ -6132,7 +6132,7 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>561</v>
@@ -6152,7 +6152,7 @@
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>564</v>
@@ -6172,7 +6172,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>567</v>
@@ -6237,7 +6237,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C6" t="s">
         <v>575</v>
@@ -6259,7 +6259,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
         <v>577</v>
@@ -6626,7 +6626,7 @@
         <v>547</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -6635,12 +6635,12 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -6649,10 +6649,10 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add companion voice notes (#32)
Occasionally (at most once every few days, gated and budgeted by the
per-open inner-life cap) a companion "records" a short spoken voice note
instead of typing. It renders as a voice-note bubble: a play/stop button,
a deterministic waveform that pulses while playing, and a show/hide
transcript toggle. Playback uses the natural voice when configured, else
browser TTS, and honors auto-speak + Calm Mode. The content reuses
proactiveCompanion via a new 'voicenote' intent, so there's no extra AI
plumbing.

- src/lib/voicenote.js: voiceNoteDue, markVoiceNote, waveform
- src/lib/ai.js: voicenote proactive intent + offline placeholder
- src/screens/Chat.jsx: inner-life voice-note beat, playVoiceNote, render branch
- docs: tracker row -> Built, regenerated xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1694,18 +1694,18 @@
     <t>NEW (task #31); lib/seasonal.js (seasonalTheme/Particles/Line/Due), occasion.js season+detectHoliday exported, CompanionSpace ambient layer + label, Chat seasonal moment effect, theme.js seasonalDrift keyframe</t>
   </si>
   <si>
+    <t>Companion voice notes</t>
+  </si>
+  <si>
+    <t>Occasionally (at most ~once every 3 days, gated) a companion 'records' a short spoken voice note instead of typing. Rendered as a voice-note bubble with a play/stop button, a seeded waveform that pulses while playing, and a show/hide transcript toggle. Plays aloud via natural voice when configured, else browser TTS; honors auto-speak + Calm Mode. Content reuses proactiveCompanion (no extra plumbing), budgeted by the per-open inner-life cap</t>
+  </si>
+  <si>
+    <t>NEW (task #32); lib/voicenote.js (voiceNoteDue/markVoiceNote/waveform), ai.js voicenote intent + placeholder, Chat inner-life beat + playVoiceNote + voicenote render branch</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>Companion voice notes</t>
-  </si>
-  <si>
-    <t>Occasional spoken messages instead of text (natural voice when configured)</t>
-  </si>
-  <si>
-    <t>PLANNED; lib/voice.js</t>
-  </si>
-  <si>
     <t>Photo moments</t>
   </si>
   <si>
@@ -1739,7 +1739,7 @@
     <t>% of total</t>
   </si>
   <si>
-    <t>90%</t>
+    <t>91%</t>
   </si>
   <si>
     <t>4%</t>
@@ -6132,27 +6132,27 @@
     </row>
     <row r="197" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B197" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="B197" s="2" t="s">
+      <c r="C197" s="2" t="s">
         <v>561</v>
       </c>
-      <c r="C197" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="D197" s="5" t="s">
-        <v>238</v>
+      <c r="D197" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="198" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>564</v>
@@ -6172,7 +6172,7 @@
     </row>
     <row r="199" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>567</v>
@@ -6237,7 +6237,7 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C6" t="s">
         <v>575</v>
@@ -6259,7 +6259,7 @@
         <v>238</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
         <v>577</v>
@@ -6388,7 +6388,7 @@
         <v>153</v>
       </c>
       <c r="B18">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -6397,7 +6397,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -6640,7 +6640,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -6649,10 +6649,10 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ambiance: let users upload their own looping sound
Adds "upload your own" to the ambiance soundscapes so users aren't
limited to the built-in synthesized ones. Any audio file (up to 20 MB)
is stored on-device in IndexedDB (not localStorage — audio is large) and
looped softly via an <audio> element. Uploads appear as selectable,
removable chips alongside the built-ins; the choice persists as a
custom:<id> key. Everything stays local — nothing is uploaded anywhere.

- src/lib/ambiance.js: IndexedDB clip store (listCustom/addCustom/
  removeCustom/getCustomBlob), isCustom, custom <audio> loop playback + cleanup
- src/screens/Settings.jsx: custom-sound chips + "Upload your own" + errors
- docs: tracker row updated, regenerated xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1874,10 +1874,10 @@
     <t>Ambiance soundscapes</t>
   </si>
   <si>
-    <t>Gentle ambient soundscapes for The Space (rain / waves / deep space / forest), synthesized live on-device with the Web Audio API — no audio files, no network. Chosen pack persists. (Full accent-theme swapping deferred: would need a design-token refactor to avoid the hex+alpha inline pattern)</t>
-  </si>
-  <si>
-    <t>NEW (task #49); lib/ambiance.js, Settings Comfort &gt; Ambiance</t>
+    <t>Gentle ambient soundscapes for The Space (rain / waves / deep space / forest) synthesized live with Web Audio, PLUS upload-your-own: any audio file (up to 20 MB) stored on-device in IndexedDB and looped softly. Chosen pack persists (custom keys are custom:&lt;id&gt;); uploads are selectable/removable chips. (Full accent-theme swapping still deferred — needs a design-token refactor)</t>
+  </si>
+  <si>
+    <t>NEW (task #49); lib/ambiance.js (Web Audio + IndexedDB custom clips), Settings Comfort &gt; Ambiance with upload</t>
   </si>
   <si>
     <t>OTHER — Feature Summary</t>

</xml_diff>

<commit_message>
Cowork: add Pomodoro focus/break timer
The Cowork station now offers two modes: a single session (25 / 50 /
Open, as before) or a Pomodoro that automatically alternates focus and
break rounds (25/5 or 50/10, repeating until you end). During a run it
shows the phase ("Focus · round N" or "☕ Break") with a break-tinted
backdrop and calmer companions; at each turn a companion posts a warm
line to chat (into a break with a tip, back to focus for the next round),
and the quiet window re-arms each cycle. The done screen tallies rounds.

Cycle math lives in a pure, unit-tested helper (lib/cowork.pomoNext).

- src/lib/cowork.js: pomoNext (verified: 25/5 and 50/10 cycles)
- src/screens/Cowork.jsx: mode toggle, pomodoro presets, phase-aware working view
- docs: tracker + regenerated xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -1715,10 +1715,10 @@
     <t>Cowork station</t>
   </si>
   <si>
-    <t>Body-doubling focus space: pick one or all awake companions, a length (25/50/Open), and a relaxing soundscape; a calming animated aurora backdrop, gentle floating companions, a soft timer + rotating encouragement, and volume control. Quiets app nudges for the session and posts a start/end line to chat. Builds on the focus + ambiance systems</t>
-  </si>
-  <si>
-    <t>NEW; screens/Cowork.jsx, Chat cowork panel + menu, startFocus/endFocus silent option</t>
+    <t>Body-doubling focus space: pick one or all awake companions, then either a single session (25/50/Open) or a Pomodoro that auto-alternates focus/break rounds (25/5 or 50/10) with round tracking and break tips. Calming animated aurora backdrop, gently floating companions, a soft timer + rotating encouragement, a relaxing soundscape + volume. Quiets app nudges and posts start/break/resume/end lines to chat</t>
+  </si>
+  <si>
+    <t>NEW; screens/Cowork.jsx + lib/cowork.pomoNext (unit-tested), Chat cowork panel + menu, startFocus/endFocus silent option</t>
   </si>
   <si>
     <t>Roadmap</t>

</xml_diff>

<commit_message>
Add a Home screen (launcher) — surfaces Cowork and everything
Features like Cowork were buried in the chat "⋯" menu. The app now opens
to a Home hub: a time-of-day greeting, today's cosmic focus, a
companion-of-the-day card, a daily check-in nudge when one's due, and big
tiles for Chat, Cowork, The Space, For you, Timeline and Settings. A 🏠
button in the chat header returns here anytime.

- src/screens/Home.jsx: the launcher
- src/screens/Chat.jsx: panel defaults to 'home', home panel route, header 🏠 button
- docs: tracker row + regenerated xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="640">
   <si>
     <t>Category</t>
   </si>
@@ -1721,6 +1721,18 @@
     <t>NEW; screens/Cowork.jsx + lib/cowork.pomoNext (unit-tested), Chat cowork panel + menu, startFocus/endFocus silent option</t>
   </si>
   <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Home screen</t>
+  </si>
+  <si>
+    <t>A landing hub the app opens to: time-of-day greeting, today's cosmic focus, companion-of-the-day, a daily check-in nudge when due, and big tiles for Chat, Cowork, The Space, For you, Timeline and Settings. A 🏠 button in the chat header returns here — so features (like Cowork) are visible instead of buried in the menu</t>
+  </si>
+  <si>
+    <t>NEW; screens/Home.jsx, Chat panel=home default + header home button</t>
+  </si>
+  <si>
     <t>Roadmap</t>
   </si>
   <si>
@@ -1892,7 +1904,7 @@
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 215 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 216 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -2364,7 +2376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F216"/>
+  <dimension ref="A1:F217"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -6365,11 +6377,11 @@
       <c r="C200" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="D200" s="5" t="s">
-        <v>238</v>
+      <c r="D200" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E200" s="2" t="s">
-        <v>313</v>
+        <v>55</v>
       </c>
       <c r="F200" s="2" t="s">
         <v>572</v>
@@ -6385,11 +6397,11 @@
       <c r="C201" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="D201" s="3" t="s">
-        <v>9</v>
+      <c r="D201" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="E201" s="2" t="s">
-        <v>55</v>
+        <v>313</v>
       </c>
       <c r="F201" s="2" t="s">
         <v>576</v>
@@ -6397,13 +6409,13 @@
     </row>
     <row r="202" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>547</v>
+        <v>577</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D202" s="3" t="s">
         <v>9</v>
@@ -6412,7 +6424,7 @@
         <v>55</v>
       </c>
       <c r="F202" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="203" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6420,19 +6432,19 @@
         <v>547</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D203" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E203" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F203" s="2" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="204" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6440,19 +6452,19 @@
         <v>547</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="D204" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F204" s="2" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="205" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6460,19 +6472,19 @@
         <v>547</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D205" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E205" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F205" s="2" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="206" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6480,10 +6492,10 @@
         <v>547</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D206" s="3" t="s">
         <v>9</v>
@@ -6492,7 +6504,7 @@
         <v>122</v>
       </c>
       <c r="F206" s="2" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="207" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6500,50 +6512,50 @@
         <v>547</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D207" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F207" s="2" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="208" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D208" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F208" s="2" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="209" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>153</v>
+        <v>540</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D209" s="3" t="s">
         <v>9</v>
@@ -6552,12 +6564,12 @@
         <v>122</v>
       </c>
       <c r="F209" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="210" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>601</v>
+        <v>153</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>602</v>
@@ -6577,13 +6589,13 @@
     </row>
     <row r="211" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>153</v>
+        <v>605</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D211" s="3" t="s">
         <v>9</v>
@@ -6592,7 +6604,7 @@
         <v>122</v>
       </c>
       <c r="F211" s="2" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="212" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6600,50 +6612,50 @@
         <v>153</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D212" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E212" s="2" t="s">
-        <v>313</v>
+        <v>122</v>
       </c>
       <c r="F212" s="2" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="213" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D213" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>122</v>
+        <v>313</v>
       </c>
       <c r="F213" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="214" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>337</v>
+        <v>109</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D214" s="3" t="s">
         <v>9</v>
@@ -6652,12 +6664,12 @@
         <v>122</v>
       </c>
       <c r="F214" s="2" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="215" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>617</v>
+        <v>337</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>618</v>
@@ -6669,7 +6681,7 @@
         <v>9</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F215" s="2" t="s">
         <v>620</v>
@@ -6689,14 +6701,34 @@
         <v>9</v>
       </c>
       <c r="E216" s="2" t="s">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="F216" s="2" t="s">
         <v>624</v>
       </c>
     </row>
+    <row r="217" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="B217" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C217" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E217" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F217" s="2" t="s">
+        <v>628</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F216"/>
+  <autoFilter ref="A1:F217"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6704,7 +6736,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -6713,17 +6745,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -6731,10 +6763,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -6742,10 +6774,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C6" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -6756,7 +6788,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -6767,23 +6799,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="B9" s="13">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -6800,7 +6832,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -7148,13 +7180,13 @@
         <v>569</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -7165,13 +7197,13 @@
         <v>573</v>
       </c>
       <c r="B34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -7179,7 +7211,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>601</v>
+        <v>577</v>
       </c>
       <c r="B35">
         <v>1</v>
@@ -7196,7 +7228,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -7225,6 +7257,23 @@
         <v>0</v>
       </c>
       <c r="E37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>625</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Companions proactively remind you about upcoming calendar events
Until now companions could only reference the calendar if it came up.
Now they bring things up unprompted — like a friend who remembered.

- lib/reminders.js: pure pickReminder over on-device events (shared
  Google events + companion-made plans/reminders). <=90 min out is an
  urgent heads-up; later-today is a gentle nudge; all-day items flag on
  the day. Each event mentioned at most once (dedup persisted, pruned).
- ai.js: new 'calendar' proactive kind — in-character reminder that
  offers to help, never sounds like a notification.
- Chat: a reminder effect (fires ~8s after open, rechecks every 3 min)
  that stays quiet during focus sessions and while the tab is hidden.

Tests: 11 new client (47 total) + a Playwright smoke proving a companion
posts a reminder for an event ~40 min out.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCbrtpGTo2snVouw3qxgtM
</commit_message>
<xml_diff>
--- a/docs/OTHER_App_Features.xlsx
+++ b/docs/OTHER_App_Features.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1413" uniqueCount="674">
   <si>
     <t>Category</t>
   </si>
@@ -1994,10 +1994,19 @@
     <t>NEW (task #51); server /calendar/enable + /calendar.ics (cal_tokens table, buildCalendarFeed VEVENTs+RRULE), api.enableCalendarFeed; 9 server tests (56 total)</t>
   </si>
   <si>
+    <t>Proactive calendar reminders</t>
+  </si>
+  <si>
+    <t>Companions bring up calendar items unprompted — like a friend who remembered — when something is coming up soon. Sources are all on-device: shared Google Calendar events and any plans/reminders a companion itself created in chat. An imminent event (&lt;=90 min) gets an urgent heads-up; something later today gets a gentle nudge; all-day items are flagged the day they arrive. Each event is mentioned at most once, and never during a focus session or while the tab is hidden</t>
+  </si>
+  <si>
+    <t>NEW (task #52); lib/reminders.js (pickReminder/whenPhrase, once-per-event dedup), ai.js 'calendar' proactive kind, Chat reminder effect over upcoming+action events; 11 client tests (47 total)</t>
+  </si>
+  <si>
     <t>OTHER — Feature Summary</t>
   </si>
   <si>
-    <t>Generated 2026-06-28 · Extratac LLC · 225 features tracked</t>
+    <t>Generated 2026-06-28 · Extratac LLC · 226 features tracked</t>
   </si>
   <si>
     <t>By status</t>
@@ -2469,7 +2478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F226"/>
+  <dimension ref="A1:F227"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -7000,8 +7009,28 @@
         <v>659</v>
       </c>
     </row>
+    <row r="227" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="B227" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E227" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F227" s="2" t="s">
+        <v>662</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F226"/>
+  <autoFilter ref="A1:F227"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -7018,17 +7047,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -7036,10 +7065,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -7047,10 +7076,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C6" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -7061,7 +7090,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -7072,23 +7101,23 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B9" s="13">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -7105,7 +7134,7 @@
         <v>238</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -7623,7 +7652,7 @@
         <v>653</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -7632,7 +7661,7 @@
         <v>0</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>